<commit_message>
Updates to PRSI Exemption reasons PIT3
</commit_message>
<xml_diff>
--- a/PIT3/Schema Publication Changelog.xlsx
+++ b/PIT3/Schema Publication Changelog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ctrowell\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sphilibi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AA6EAA-E12C-4619-95BB-7FF0D0ACF732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58FF0AF2-D6B1-4E63-9978-B240AB24CB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-210" yWindow="0" windowWidth="21600" windowHeight="15600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19080" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v0.10" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Walsh, David P - Personal View" guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1436" windowHeight="675" activeSheetId="2"/>
+    <customWorkbookView name="Arnold, Eve - Personal View" guid="{057DBB0B-BBF6-4A94-8406-46C99A7DC1D6}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="758" activeSheetId="2"/>
     <customWorkbookView name="O'Brien, Ciaran - Personal View" guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="751" activeSheetId="2"/>
-    <customWorkbookView name="Arnold, Eve - Personal View" guid="{057DBB0B-BBF6-4A94-8406-46C99A7DC1D6}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="758" activeSheetId="2"/>
-    <customWorkbookView name="Walsh, David P - Personal View" guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1436" windowHeight="675" activeSheetId="2"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="586">
   <si>
     <t>Document</t>
   </si>
@@ -3625,12 +3625,27 @@
   <si>
     <t>ERR - Enhanced Reporting Submission Request Data Items</t>
   </si>
+  <si>
+    <t>PRSI Exemption Reason Updates</t>
+  </si>
+  <si>
+    <t>Payroll Employer Submission - Employee Level Validation</t>
+  </si>
+  <si>
+    <t>PIT Next Version</t>
+  </si>
+  <si>
+    <t>PRSI Class and Subclass</t>
+  </si>
+  <si>
+    <t>Warning added on PRSI Class and Subclass</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3777,6 +3792,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -4238,7 +4259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="263">
+  <cellXfs count="268">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -4710,6 +4731,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -4755,8 +4779,38 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -4779,66 +4833,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4860,25 +4854,103 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4890,71 +4962,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5320,12 +5354,12 @@
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="181" t="s">
+      <c r="A2" s="182" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="182"/>
-      <c r="C2" s="182"/>
-      <c r="D2" s="183"/>
+      <c r="B2" s="183"/>
+      <c r="C2" s="183"/>
+      <c r="D2" s="184"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -5348,12 +5382,12 @@
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="181" t="s">
+      <c r="A4" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="182"/>
-      <c r="C4" s="182"/>
-      <c r="D4" s="183"/>
+      <c r="B4" s="183"/>
+      <c r="C4" s="183"/>
+      <c r="D4" s="184"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -5393,10 +5427,10 @@
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="184" t="s">
+      <c r="A7" s="185" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="187">
+      <c r="B7" s="188">
         <v>0.1</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -5410,8 +5444,8 @@
       <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="185"/>
-      <c r="B8" s="188"/>
+      <c r="A8" s="186"/>
+      <c r="B8" s="189"/>
       <c r="C8" s="11" t="s">
         <v>5</v>
       </c>
@@ -5423,8 +5457,8 @@
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="185"/>
-      <c r="B9" s="188"/>
+      <c r="A9" s="186"/>
+      <c r="B9" s="189"/>
       <c r="C9" s="11" t="s">
         <v>6</v>
       </c>
@@ -5436,8 +5470,8 @@
       <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="185"/>
-      <c r="B10" s="188"/>
+      <c r="A10" s="186"/>
+      <c r="B10" s="189"/>
       <c r="C10" s="11" t="s">
         <v>61</v>
       </c>
@@ -5449,8 +5483,8 @@
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="185"/>
-      <c r="B11" s="188"/>
+      <c r="A11" s="186"/>
+      <c r="B11" s="189"/>
       <c r="C11" s="11" t="s">
         <v>73</v>
       </c>
@@ -5462,8 +5496,8 @@
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="186"/>
-      <c r="B12" s="189"/>
+      <c r="A12" s="187"/>
+      <c r="B12" s="190"/>
       <c r="C12" s="11" t="s">
         <v>67</v>
       </c>
@@ -5475,10 +5509,10 @@
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="192" t="s">
+      <c r="A13" s="193" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="187">
+      <c r="B13" s="188">
         <v>0.1</v>
       </c>
       <c r="C13" s="11" t="s">
@@ -5492,8 +5526,8 @@
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="193"/>
-      <c r="B14" s="189"/>
+      <c r="A14" s="194"/>
+      <c r="B14" s="190"/>
       <c r="C14" s="11" t="s">
         <v>69</v>
       </c>
@@ -5539,12 +5573,12 @@
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="181" t="s">
+      <c r="A17" s="182" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="182"/>
-      <c r="C17" s="182"/>
-      <c r="D17" s="183"/>
+      <c r="B17" s="183"/>
+      <c r="C17" s="183"/>
+      <c r="D17" s="184"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -5584,21 +5618,21 @@
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="181" t="s">
+      <c r="A20" s="182" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="182"/>
-      <c r="C20" s="182"/>
-      <c r="D20" s="183"/>
+      <c r="B20" s="183"/>
+      <c r="C20" s="183"/>
+      <c r="D20" s="184"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
     <row r="21" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="194" t="s">
+      <c r="A21" s="195" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="191">
+      <c r="B21" s="192">
         <v>0.1</v>
       </c>
       <c r="C21" s="11" t="s">
@@ -5612,8 +5646,8 @@
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="195"/>
-      <c r="B22" s="189"/>
+      <c r="A22" s="196"/>
+      <c r="B22" s="190"/>
       <c r="C22" s="27" t="s">
         <v>37</v>
       </c>
@@ -5636,18 +5670,18 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="181" t="s">
+      <c r="A24" s="182" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="182"/>
-      <c r="C24" s="182"/>
-      <c r="D24" s="183"/>
+      <c r="B24" s="183"/>
+      <c r="C24" s="183"/>
+      <c r="D24" s="184"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="190" t="s">
+      <c r="A25" s="191" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="191">
+      <c r="B25" s="192">
         <v>0.1</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -5661,8 +5695,8 @@
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="185"/>
-      <c r="B26" s="188"/>
+      <c r="A26" s="186"/>
+      <c r="B26" s="189"/>
       <c r="C26" s="11" t="s">
         <v>71</v>
       </c>
@@ -5674,8 +5708,8 @@
       <c r="G26" s="2"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="185"/>
-      <c r="B27" s="188"/>
+      <c r="A27" s="186"/>
+      <c r="B27" s="189"/>
       <c r="C27" s="11" t="s">
         <v>11</v>
       </c>
@@ -5687,8 +5721,8 @@
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A28" s="185"/>
-      <c r="B28" s="188"/>
+      <c r="A28" s="186"/>
+      <c r="B28" s="189"/>
       <c r="C28" s="21" t="s">
         <v>72</v>
       </c>
@@ -5700,8 +5734,8 @@
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="185"/>
-      <c r="B29" s="188"/>
+      <c r="A29" s="186"/>
+      <c r="B29" s="189"/>
       <c r="C29" s="11" t="s">
         <v>9</v>
       </c>
@@ -5713,8 +5747,8 @@
       <c r="G29" s="2"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="185"/>
-      <c r="B30" s="188"/>
+      <c r="A30" s="186"/>
+      <c r="B30" s="189"/>
       <c r="C30" s="11" t="s">
         <v>13</v>
       </c>
@@ -5726,8 +5760,8 @@
       <c r="G30" s="2"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="185"/>
-      <c r="B31" s="188"/>
+      <c r="A31" s="186"/>
+      <c r="B31" s="189"/>
       <c r="C31" s="11" t="s">
         <v>15</v>
       </c>
@@ -5739,8 +5773,8 @@
       <c r="G31" s="2"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="186"/>
-      <c r="B32" s="189"/>
+      <c r="A32" s="187"/>
+      <c r="B32" s="190"/>
       <c r="C32" s="11" t="s">
         <v>17</v>
       </c>
@@ -5864,12 +5898,12 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="181" t="s">
+      <c r="A41" s="182" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="182"/>
-      <c r="C41" s="182"/>
-      <c r="D41" s="183"/>
+      <c r="B41" s="183"/>
+      <c r="C41" s="183"/>
+      <c r="D41" s="184"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
@@ -5929,7 +5963,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="B1">
+    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}" topLeftCell="B1">
       <selection activeCell="C15" sqref="C15:D15"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5939,7 +5973,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
     </customSheetView>
-    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}" topLeftCell="B1">
+    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="B1">
       <selection activeCell="C15" sqref="C15:D15"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
@@ -6044,10 +6078,10 @@
       <c r="D6" s="44"/>
     </row>
     <row r="7" spans="1:4" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="211" t="s">
+      <c r="A7" s="197" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="210" t="s">
+      <c r="B7" s="198" t="s">
         <v>85</v>
       </c>
       <c r="C7" s="43" t="s">
@@ -6058,8 +6092,8 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="211"/>
-      <c r="B8" s="210"/>
+      <c r="A8" s="197"/>
+      <c r="B8" s="198"/>
       <c r="C8" s="38" t="s">
         <v>88</v>
       </c>
@@ -6068,8 +6102,8 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="211"/>
-      <c r="B9" s="210"/>
+      <c r="A9" s="197"/>
+      <c r="B9" s="198"/>
       <c r="C9" s="38" t="s">
         <v>89</v>
       </c>
@@ -6078,8 +6112,8 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="211"/>
-      <c r="B10" s="210"/>
+      <c r="A10" s="197"/>
+      <c r="B10" s="198"/>
       <c r="C10" s="38" t="s">
         <v>6</v>
       </c>
@@ -6088,8 +6122,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="211"/>
-      <c r="B11" s="210"/>
+      <c r="A11" s="197"/>
+      <c r="B11" s="198"/>
       <c r="C11" s="38" t="s">
         <v>93</v>
       </c>
@@ -6098,8 +6132,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="211"/>
-      <c r="B12" s="210"/>
+      <c r="A12" s="197"/>
+      <c r="B12" s="198"/>
       <c r="C12" s="38" t="s">
         <v>96</v>
       </c>
@@ -6108,10 +6142,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="213" t="s">
+      <c r="A13" s="200" t="s">
         <v>146</v>
       </c>
-      <c r="B13" s="210" t="s">
+      <c r="B13" s="198" t="s">
         <v>85</v>
       </c>
       <c r="C13" s="38" t="s">
@@ -6122,8 +6156,8 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="213"/>
-      <c r="B14" s="210"/>
+      <c r="A14" s="200"/>
+      <c r="B14" s="198"/>
       <c r="C14" s="38" t="s">
         <v>180</v>
       </c>
@@ -6132,8 +6166,8 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="213"/>
-      <c r="B15" s="210"/>
+      <c r="A15" s="200"/>
+      <c r="B15" s="198"/>
       <c r="C15" s="43" t="s">
         <v>182</v>
       </c>
@@ -6142,10 +6176,10 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="196" t="s">
+      <c r="A16" s="201" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="205" t="s">
+      <c r="B16" s="202" t="s">
         <v>85</v>
       </c>
       <c r="C16" s="59" t="s">
@@ -6156,8 +6190,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="196"/>
-      <c r="B17" s="205"/>
+      <c r="A17" s="201"/>
+      <c r="B17" s="202"/>
       <c r="C17" s="58" t="s">
         <v>148</v>
       </c>
@@ -6166,8 +6200,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="196"/>
-      <c r="B18" s="205"/>
+      <c r="A18" s="201"/>
+      <c r="B18" s="202"/>
       <c r="C18" s="58" t="s">
         <v>93</v>
       </c>
@@ -6176,8 +6210,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="196"/>
-      <c r="B19" s="205"/>
+      <c r="A19" s="201"/>
+      <c r="B19" s="202"/>
       <c r="C19" s="58" t="s">
         <v>151</v>
       </c>
@@ -6186,8 +6220,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="196"/>
-      <c r="B20" s="205"/>
+      <c r="A20" s="201"/>
+      <c r="B20" s="202"/>
       <c r="C20" s="58" t="s">
         <v>153</v>
       </c>
@@ -6196,8 +6230,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="196"/>
-      <c r="B21" s="205"/>
+      <c r="A21" s="201"/>
+      <c r="B21" s="202"/>
       <c r="C21" s="58" t="s">
         <v>155</v>
       </c>
@@ -6206,8 +6240,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="196"/>
-      <c r="B22" s="205"/>
+      <c r="A22" s="201"/>
+      <c r="B22" s="202"/>
       <c r="C22" s="58" t="s">
         <v>157</v>
       </c>
@@ -6216,8 +6250,8 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="196"/>
-      <c r="B23" s="205"/>
+      <c r="A23" s="201"/>
+      <c r="B23" s="202"/>
       <c r="C23" s="66" t="s">
         <v>159</v>
       </c>
@@ -6226,26 +6260,26 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="196"/>
-      <c r="B24" s="205"/>
-      <c r="C24" s="196" t="s">
+      <c r="A24" s="201"/>
+      <c r="B24" s="202"/>
+      <c r="C24" s="201" t="s">
         <v>161</v>
       </c>
-      <c r="D24" s="197" t="s">
+      <c r="D24" s="208" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="196"/>
-      <c r="B25" s="205"/>
-      <c r="C25" s="196"/>
-      <c r="D25" s="197"/>
+      <c r="A25" s="201"/>
+      <c r="B25" s="202"/>
+      <c r="C25" s="201"/>
+      <c r="D25" s="208"/>
     </row>
     <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="211" t="s">
+      <c r="A26" s="197" t="s">
         <v>163</v>
       </c>
-      <c r="B26" s="210" t="s">
+      <c r="B26" s="198" t="s">
         <v>85</v>
       </c>
       <c r="C26" s="38" t="s">
@@ -6256,8 +6290,8 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="211"/>
-      <c r="B27" s="210"/>
+      <c r="A27" s="197"/>
+      <c r="B27" s="198"/>
       <c r="C27" s="38"/>
       <c r="D27" s="41" t="s">
         <v>118</v>
@@ -6284,28 +6318,28 @@
       <c r="D29" s="39"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="212" t="s">
+      <c r="A30" s="199" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="210" t="s">
+      <c r="B30" s="198" t="s">
         <v>85</v>
       </c>
-      <c r="C30" s="196" t="s">
+      <c r="C30" s="201" t="s">
         <v>169</v>
       </c>
-      <c r="D30" s="200" t="s">
+      <c r="D30" s="211" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="212"/>
-      <c r="B31" s="210"/>
-      <c r="C31" s="196"/>
-      <c r="D31" s="200"/>
+      <c r="A31" s="199"/>
+      <c r="B31" s="198"/>
+      <c r="C31" s="201"/>
+      <c r="D31" s="211"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="212"/>
-      <c r="B32" s="210"/>
+      <c r="A32" s="199"/>
+      <c r="B32" s="198"/>
       <c r="C32" s="58" t="s">
         <v>167</v>
       </c>
@@ -6314,8 +6348,8 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="212"/>
-      <c r="B33" s="210"/>
+      <c r="A33" s="199"/>
+      <c r="B33" s="198"/>
       <c r="C33" s="58" t="s">
         <v>168</v>
       </c>
@@ -6324,8 +6358,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="212"/>
-      <c r="B34" s="210"/>
+      <c r="A34" s="199"/>
+      <c r="B34" s="198"/>
       <c r="C34" s="67" t="s">
         <v>170</v>
       </c>
@@ -6334,8 +6368,8 @@
       </c>
     </row>
     <row r="35" spans="1:4" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="212"/>
-      <c r="B35" s="210"/>
+      <c r="A35" s="199"/>
+      <c r="B35" s="198"/>
       <c r="C35" s="58" t="s">
         <v>157</v>
       </c>
@@ -6344,8 +6378,8 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="212"/>
-      <c r="B36" s="210"/>
+      <c r="A36" s="199"/>
+      <c r="B36" s="198"/>
       <c r="C36" s="67" t="s">
         <v>159</v>
       </c>
@@ -6354,26 +6388,26 @@
       </c>
     </row>
     <row r="37" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="212"/>
-      <c r="B37" s="210"/>
-      <c r="C37" s="201" t="s">
+      <c r="A37" s="199"/>
+      <c r="B37" s="198"/>
+      <c r="C37" s="212" t="s">
         <v>161</v>
       </c>
-      <c r="D37" s="203" t="s">
+      <c r="D37" s="214" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="6.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="212"/>
-      <c r="B38" s="210"/>
-      <c r="C38" s="202"/>
-      <c r="D38" s="203"/>
+      <c r="A38" s="199"/>
+      <c r="B38" s="198"/>
+      <c r="C38" s="213"/>
+      <c r="D38" s="214"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="211" t="s">
+      <c r="A39" s="197" t="s">
         <v>86</v>
       </c>
-      <c r="B39" s="210" t="s">
+      <c r="B39" s="198" t="s">
         <v>85</v>
       </c>
       <c r="C39" s="38" t="s">
@@ -6384,8 +6418,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="211"/>
-      <c r="B40" s="210"/>
+      <c r="A40" s="197"/>
+      <c r="B40" s="198"/>
       <c r="C40" s="38"/>
       <c r="D40" s="49" t="s">
         <v>98</v>
@@ -6412,10 +6446,10 @@
       <c r="D42" s="44"/>
     </row>
     <row r="43" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="212" t="s">
+      <c r="A43" s="199" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="210" t="s">
+      <c r="B43" s="198" t="s">
         <v>85</v>
       </c>
       <c r="C43" s="38"/>
@@ -6424,8 +6458,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="212"/>
-      <c r="B44" s="210"/>
+      <c r="A44" s="199"/>
+      <c r="B44" s="198"/>
       <c r="C44" s="38" t="s">
         <v>145</v>
       </c>
@@ -6434,10 +6468,10 @@
       </c>
     </row>
     <row r="45" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="207" t="s">
+      <c r="A45" s="205" t="s">
         <v>80</v>
       </c>
-      <c r="B45" s="210" t="s">
+      <c r="B45" s="198" t="s">
         <v>85</v>
       </c>
       <c r="C45" s="38"/>
@@ -6446,8 +6480,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="208"/>
-      <c r="B46" s="210"/>
+      <c r="A46" s="206"/>
+      <c r="B46" s="198"/>
       <c r="C46" s="38" t="s">
         <v>101</v>
       </c>
@@ -6456,8 +6490,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="208"/>
-      <c r="B47" s="210"/>
+      <c r="A47" s="206"/>
+      <c r="B47" s="198"/>
       <c r="C47" s="38" t="s">
         <v>99</v>
       </c>
@@ -6466,8 +6500,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="209"/>
-      <c r="B48" s="210"/>
+      <c r="A48" s="207"/>
+      <c r="B48" s="198"/>
       <c r="C48" s="38" t="s">
         <v>145</v>
       </c>
@@ -6476,10 +6510,10 @@
       </c>
     </row>
     <row r="49" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A49" s="205" t="s">
+      <c r="A49" s="202" t="s">
         <v>32</v>
       </c>
-      <c r="B49" s="205" t="s">
+      <c r="B49" s="202" t="s">
         <v>85</v>
       </c>
       <c r="C49" s="58"/>
@@ -10583,8 +10617,8 @@
       <c r="XFC49" s="42"/>
     </row>
     <row r="50" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="205"/>
-      <c r="B50" s="205"/>
+      <c r="A50" s="202"/>
+      <c r="B50" s="202"/>
       <c r="C50" s="59" t="s">
         <v>105</v>
       </c>
@@ -14688,8 +14722,8 @@
       <c r="XFC50" s="42"/>
     </row>
     <row r="51" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A51" s="205"/>
-      <c r="B51" s="205"/>
+      <c r="A51" s="202"/>
+      <c r="B51" s="202"/>
       <c r="C51" s="38" t="s">
         <v>107</v>
       </c>
@@ -18793,8 +18827,8 @@
       <c r="XFC51" s="42"/>
     </row>
     <row r="52" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A52" s="205"/>
-      <c r="B52" s="205"/>
+      <c r="A52" s="202"/>
+      <c r="B52" s="202"/>
       <c r="C52" s="58" t="s">
         <v>108</v>
       </c>
@@ -22898,12 +22932,12 @@
       <c r="XFC52" s="42"/>
     </row>
     <row r="53" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A53" s="205"/>
-      <c r="B53" s="205"/>
-      <c r="C53" s="199" t="s">
+      <c r="A53" s="202"/>
+      <c r="B53" s="202"/>
+      <c r="C53" s="210" t="s">
         <v>109</v>
       </c>
-      <c r="D53" s="200" t="s">
+      <c r="D53" s="211" t="s">
         <v>144</v>
       </c>
       <c r="G53" s="42"/>
@@ -27003,10 +27037,10 @@
       <c r="XFC53" s="42"/>
     </row>
     <row r="54" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="205"/>
-      <c r="B54" s="205"/>
-      <c r="C54" s="199"/>
-      <c r="D54" s="200"/>
+      <c r="A54" s="202"/>
+      <c r="B54" s="202"/>
+      <c r="C54" s="210"/>
+      <c r="D54" s="211"/>
       <c r="G54" s="42"/>
       <c r="K54" s="42"/>
       <c r="O54" s="42"/>
@@ -31124,10 +31158,10 @@
       </c>
     </row>
     <row r="57" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A57" s="204" t="s">
+      <c r="A57" s="203" t="s">
         <v>84</v>
       </c>
-      <c r="B57" s="205" t="s">
+      <c r="B57" s="202" t="s">
         <v>85</v>
       </c>
       <c r="C57" s="58" t="s">
@@ -31138,8 +31172,8 @@
       </c>
     </row>
     <row r="58" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="204"/>
-      <c r="B58" s="205"/>
+      <c r="A58" s="203"/>
+      <c r="B58" s="202"/>
       <c r="C58" s="61" t="s">
         <v>113</v>
       </c>
@@ -31148,8 +31182,8 @@
       </c>
     </row>
     <row r="59" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A59" s="204"/>
-      <c r="B59" s="205"/>
+      <c r="A59" s="203"/>
+      <c r="B59" s="202"/>
       <c r="C59" s="58" t="s">
         <v>114</v>
       </c>
@@ -31158,8 +31192,8 @@
       </c>
     </row>
     <row r="60" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="30" x14ac:dyDescent="0.25">
-      <c r="A60" s="204"/>
-      <c r="B60" s="205"/>
+      <c r="A60" s="203"/>
+      <c r="B60" s="202"/>
       <c r="C60" s="58" t="s">
         <v>115</v>
       </c>
@@ -31168,8 +31202,8 @@
       </c>
     </row>
     <row r="61" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A61" s="204"/>
-      <c r="B61" s="205"/>
+      <c r="A61" s="203"/>
+      <c r="B61" s="202"/>
       <c r="C61" s="38" t="s">
         <v>145</v>
       </c>
@@ -31178,8 +31212,8 @@
       </c>
     </row>
     <row r="62" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A62" s="204"/>
-      <c r="B62" s="205"/>
+      <c r="A62" s="203"/>
+      <c r="B62" s="202"/>
       <c r="C62" s="58" t="s">
         <v>117</v>
       </c>
@@ -31188,8 +31222,8 @@
       </c>
     </row>
     <row r="63" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A63" s="204"/>
-      <c r="B63" s="205"/>
+      <c r="A63" s="203"/>
+      <c r="B63" s="202"/>
       <c r="C63" s="58" t="s">
         <v>117</v>
       </c>
@@ -31198,16 +31232,16 @@
       </c>
     </row>
     <row r="64" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A64" s="204"/>
-      <c r="B64" s="205"/>
+      <c r="A64" s="203"/>
+      <c r="B64" s="202"/>
       <c r="C64" s="58"/>
       <c r="D64" s="47" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="204"/>
-      <c r="B65" s="205"/>
+      <c r="A65" s="203"/>
+      <c r="B65" s="202"/>
       <c r="C65" s="58" t="s">
         <v>120</v>
       </c>
@@ -31216,16 +31250,16 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="204"/>
-      <c r="B66" s="205"/>
+      <c r="A66" s="203"/>
+      <c r="B66" s="202"/>
       <c r="C66" s="58"/>
       <c r="D66" s="46" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="204"/>
-      <c r="B67" s="205"/>
+      <c r="A67" s="203"/>
+      <c r="B67" s="202"/>
       <c r="C67" s="58" t="s">
         <v>122</v>
       </c>
@@ -31234,8 +31268,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A68" s="204"/>
-      <c r="B68" s="205"/>
+      <c r="A68" s="203"/>
+      <c r="B68" s="202"/>
       <c r="C68" s="58" t="s">
         <v>123</v>
       </c>
@@ -31244,8 +31278,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A69" s="204"/>
-      <c r="B69" s="205"/>
+      <c r="A69" s="203"/>
+      <c r="B69" s="202"/>
       <c r="C69" s="61" t="s">
         <v>125</v>
       </c>
@@ -31254,8 +31288,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A70" s="204"/>
-      <c r="B70" s="205"/>
+      <c r="A70" s="203"/>
+      <c r="B70" s="202"/>
       <c r="C70" s="61" t="s">
         <v>126</v>
       </c>
@@ -31264,8 +31298,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="204"/>
-      <c r="B71" s="205"/>
+      <c r="A71" s="203"/>
+      <c r="B71" s="202"/>
       <c r="C71" s="58" t="s">
         <v>127</v>
       </c>
@@ -31274,8 +31308,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="204"/>
-      <c r="B72" s="205"/>
+      <c r="A72" s="203"/>
+      <c r="B72" s="202"/>
       <c r="C72" s="58" t="s">
         <v>128</v>
       </c>
@@ -31284,16 +31318,16 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="204"/>
-      <c r="B73" s="205"/>
+      <c r="A73" s="203"/>
+      <c r="B73" s="202"/>
       <c r="C73" s="58"/>
       <c r="D73" s="49" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="204"/>
-      <c r="B74" s="205"/>
+      <c r="A74" s="203"/>
+      <c r="B74" s="202"/>
       <c r="C74" s="58" t="s">
         <v>129</v>
       </c>
@@ -31302,18 +31336,18 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="204"/>
-      <c r="B75" s="205"/>
-      <c r="C75" s="198"/>
-      <c r="D75" s="206" t="s">
+      <c r="A75" s="203"/>
+      <c r="B75" s="202"/>
+      <c r="C75" s="209"/>
+      <c r="D75" s="204" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="204"/>
-      <c r="B76" s="205"/>
-      <c r="C76" s="198"/>
-      <c r="D76" s="206"/>
+      <c r="A76" s="203"/>
+      <c r="B76" s="202"/>
+      <c r="C76" s="209"/>
+      <c r="D76" s="204"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="39" t="s">
@@ -31337,8 +31371,8 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="A13">
-      <selection activeCell="D20" sqref="D20"/>
+    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}">
+      <selection activeCell="A7" sqref="A7"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
     </customSheetView>
@@ -31347,13 +31381,29 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
     </customSheetView>
-    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}">
-      <selection activeCell="A7" sqref="A7"/>
+    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="A13">
+      <selection activeCell="D20" sqref="D20"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="30">
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="A57:A76"/>
+    <mergeCell ref="B57:B76"/>
+    <mergeCell ref="D75:D76"/>
+    <mergeCell ref="A45:A48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="B49:B54"/>
     <mergeCell ref="A7:A12"/>
     <mergeCell ref="B7:B12"/>
     <mergeCell ref="A43:A44"/>
@@ -31368,22 +31418,6 @@
     <mergeCell ref="B16:B25"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="B39:B40"/>
-    <mergeCell ref="A57:A76"/>
-    <mergeCell ref="B57:B76"/>
-    <mergeCell ref="D75:D76"/>
-    <mergeCell ref="A45:A48"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="B49:B54"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
@@ -31432,10 +31466,10 @@
       <c r="D3" s="44"/>
     </row>
     <row r="4" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="211" t="s">
+      <c r="A4" s="197" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="210" t="s">
+      <c r="B4" s="198" t="s">
         <v>185</v>
       </c>
       <c r="C4" s="72" t="s">
@@ -31446,133 +31480,133 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="211"/>
-      <c r="B5" s="210"/>
-      <c r="C5" s="221" t="s">
+      <c r="A5" s="197"/>
+      <c r="B5" s="198"/>
+      <c r="C5" s="224" t="s">
         <v>190</v>
       </c>
-      <c r="D5" s="220" t="s">
+      <c r="D5" s="223" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="7.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="211"/>
-      <c r="B6" s="210"/>
-      <c r="C6" s="221"/>
-      <c r="D6" s="220"/>
+      <c r="A6" s="197"/>
+      <c r="B6" s="198"/>
+      <c r="C6" s="224"/>
+      <c r="D6" s="223"/>
     </row>
     <row r="7" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="211"/>
-      <c r="B7" s="210"/>
+      <c r="A7" s="197"/>
+      <c r="B7" s="198"/>
       <c r="C7" s="58"/>
       <c r="D7" s="58"/>
     </row>
     <row r="8" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="211"/>
-      <c r="B8" s="210"/>
+      <c r="A8" s="197"/>
+      <c r="B8" s="198"/>
       <c r="C8" s="58"/>
       <c r="D8" s="58"/>
     </row>
     <row r="9" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="211"/>
-      <c r="B9" s="210"/>
+      <c r="A9" s="197"/>
+      <c r="B9" s="198"/>
       <c r="C9" s="71"/>
       <c r="D9" s="49"/>
     </row>
     <row r="10" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="213" t="s">
+      <c r="A10" s="200" t="s">
         <v>146</v>
       </c>
-      <c r="B10" s="210" t="s">
+      <c r="B10" s="198" t="s">
         <v>185</v>
       </c>
-      <c r="C10" s="223"/>
-      <c r="D10" s="220" t="s">
+      <c r="C10" s="222"/>
+      <c r="D10" s="223" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="213"/>
-      <c r="B11" s="210"/>
-      <c r="C11" s="223"/>
-      <c r="D11" s="220"/>
+      <c r="A11" s="200"/>
+      <c r="B11" s="198"/>
+      <c r="C11" s="222"/>
+      <c r="D11" s="223"/>
     </row>
     <row r="12" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="213"/>
-      <c r="B12" s="210"/>
-      <c r="C12" s="223"/>
-      <c r="D12" s="220"/>
+      <c r="A12" s="200"/>
+      <c r="B12" s="198"/>
+      <c r="C12" s="222"/>
+      <c r="D12" s="223"/>
     </row>
     <row r="13" spans="1:4" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="196" t="s">
+      <c r="A13" s="201" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="205" t="s">
+      <c r="B13" s="202" t="s">
         <v>185</v>
       </c>
-      <c r="C13" s="222"/>
-      <c r="D13" s="220" t="s">
+      <c r="C13" s="225"/>
+      <c r="D13" s="223" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="196"/>
-      <c r="B14" s="205"/>
-      <c r="C14" s="222"/>
-      <c r="D14" s="220"/>
+      <c r="A14" s="201"/>
+      <c r="B14" s="202"/>
+      <c r="C14" s="225"/>
+      <c r="D14" s="223"/>
     </row>
     <row r="15" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="196"/>
-      <c r="B15" s="205"/>
-      <c r="C15" s="222"/>
+      <c r="A15" s="201"/>
+      <c r="B15" s="202"/>
+      <c r="C15" s="225"/>
       <c r="D15" s="49"/>
     </row>
     <row r="16" spans="1:4" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="196"/>
-      <c r="B16" s="205"/>
-      <c r="C16" s="222"/>
+      <c r="A16" s="201"/>
+      <c r="B16" s="202"/>
+      <c r="C16" s="225"/>
       <c r="D16" s="49"/>
     </row>
     <row r="17" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="196"/>
-      <c r="B17" s="205"/>
-      <c r="C17" s="222"/>
+      <c r="A17" s="201"/>
+      <c r="B17" s="202"/>
+      <c r="C17" s="225"/>
       <c r="D17" s="49"/>
     </row>
     <row r="18" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="196"/>
-      <c r="B18" s="205"/>
-      <c r="C18" s="222"/>
+      <c r="A18" s="201"/>
+      <c r="B18" s="202"/>
+      <c r="C18" s="225"/>
       <c r="D18" s="49"/>
     </row>
     <row r="19" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="196"/>
-      <c r="B19" s="205"/>
-      <c r="C19" s="222"/>
+      <c r="A19" s="201"/>
+      <c r="B19" s="202"/>
+      <c r="C19" s="225"/>
       <c r="D19" s="49"/>
     </row>
     <row r="20" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="196"/>
-      <c r="B20" s="205"/>
-      <c r="C20" s="222"/>
+      <c r="A20" s="201"/>
+      <c r="B20" s="202"/>
+      <c r="C20" s="225"/>
       <c r="D20" s="49"/>
     </row>
     <row r="21" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="196"/>
-      <c r="B21" s="205"/>
-      <c r="C21" s="222"/>
+      <c r="A21" s="201"/>
+      <c r="B21" s="202"/>
+      <c r="C21" s="225"/>
       <c r="D21" s="49"/>
     </row>
     <row r="22" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="196"/>
-      <c r="B22" s="205"/>
-      <c r="C22" s="222"/>
+      <c r="A22" s="201"/>
+      <c r="B22" s="202"/>
+      <c r="C22" s="225"/>
       <c r="D22" s="49"/>
     </row>
     <row r="23" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="196"/>
-      <c r="B23" s="205"/>
-      <c r="C23" s="222"/>
+      <c r="A23" s="201"/>
+      <c r="B23" s="202"/>
+      <c r="C23" s="225"/>
       <c r="D23" s="58" t="s">
         <v>221</v>
       </c>
@@ -31670,10 +31704,10 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="214" t="s">
+      <c r="A32" s="226" t="s">
         <v>222</v>
       </c>
-      <c r="B32" s="217" t="s">
+      <c r="B32" s="229" t="s">
         <v>185</v>
       </c>
       <c r="C32" s="91" t="s">
@@ -31684,26 +31718,26 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="215"/>
-      <c r="B33" s="218"/>
+      <c r="A33" s="227"/>
+      <c r="B33" s="230"/>
       <c r="C33" s="78"/>
       <c r="D33" s="75"/>
     </row>
     <row r="34" spans="1:4" ht="9.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="215"/>
-      <c r="B34" s="218"/>
+      <c r="A34" s="227"/>
+      <c r="B34" s="230"/>
       <c r="C34" s="78"/>
       <c r="D34" s="75"/>
     </row>
     <row r="35" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="215"/>
-      <c r="B35" s="218"/>
+      <c r="A35" s="227"/>
+      <c r="B35" s="230"/>
       <c r="C35" s="78"/>
       <c r="D35" s="75"/>
     </row>
     <row r="36" spans="1:4" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="216"/>
-      <c r="B36" s="219"/>
+      <c r="A36" s="228"/>
+      <c r="B36" s="231"/>
       <c r="C36" s="78" t="s">
         <v>223</v>
       </c>
@@ -31732,10 +31766,10 @@
       <c r="D38" s="44"/>
     </row>
     <row r="39" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="212" t="s">
+      <c r="A39" s="199" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="210" t="s">
+      <c r="B39" s="198" t="s">
         <v>185</v>
       </c>
       <c r="C39" s="76" t="s">
@@ -31746,8 +31780,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="212"/>
-      <c r="B40" s="210"/>
+      <c r="A40" s="199"/>
+      <c r="B40" s="198"/>
       <c r="C40" s="69" t="s">
         <v>190</v>
       </c>
@@ -31756,84 +31790,84 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="211" t="s">
+      <c r="A41" s="197" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="210" t="s">
+      <c r="B41" s="198" t="s">
         <v>185</v>
       </c>
-      <c r="C41" s="223" t="s">
+      <c r="C41" s="222" t="s">
         <v>194</v>
       </c>
-      <c r="D41" s="196" t="s">
+      <c r="D41" s="201" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="211"/>
-      <c r="B42" s="210"/>
-      <c r="C42" s="223"/>
-      <c r="D42" s="196"/>
+      <c r="A42" s="197"/>
+      <c r="B42" s="198"/>
+      <c r="C42" s="222"/>
+      <c r="D42" s="201"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="211"/>
-      <c r="B43" s="210"/>
-      <c r="C43" s="223" t="s">
+      <c r="A43" s="197"/>
+      <c r="B43" s="198"/>
+      <c r="C43" s="222" t="s">
         <v>190</v>
       </c>
-      <c r="D43" s="206" t="s">
+      <c r="D43" s="204" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="211"/>
-      <c r="B44" s="210"/>
-      <c r="C44" s="223"/>
-      <c r="D44" s="206"/>
+      <c r="A44" s="197"/>
+      <c r="B44" s="198"/>
+      <c r="C44" s="222"/>
+      <c r="D44" s="204"/>
     </row>
     <row r="45" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="204" t="s">
+      <c r="A45" s="203" t="s">
         <v>32</v>
       </c>
-      <c r="B45" s="205" t="s">
+      <c r="B45" s="202" t="s">
         <v>185</v>
       </c>
-      <c r="C45" s="227"/>
+      <c r="C45" s="218"/>
       <c r="D45" s="90" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="204"/>
-      <c r="B46" s="205"/>
-      <c r="C46" s="228"/>
-      <c r="D46" s="224" t="s">
+      <c r="A46" s="203"/>
+      <c r="B46" s="202"/>
+      <c r="C46" s="219"/>
+      <c r="D46" s="215" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="204"/>
-      <c r="B47" s="205"/>
-      <c r="C47" s="228"/>
-      <c r="D47" s="225"/>
+      <c r="A47" s="203"/>
+      <c r="B47" s="202"/>
+      <c r="C47" s="219"/>
+      <c r="D47" s="216"/>
     </row>
     <row r="48" spans="1:4" ht="13.9" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="204"/>
-      <c r="B48" s="205"/>
-      <c r="C48" s="229"/>
-      <c r="D48" s="225"/>
+      <c r="A48" s="203"/>
+      <c r="B48" s="202"/>
+      <c r="C48" s="220"/>
+      <c r="D48" s="216"/>
     </row>
     <row r="49" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="204"/>
-      <c r="B49" s="205"/>
-      <c r="C49" s="199"/>
-      <c r="D49" s="225"/>
+      <c r="A49" s="203"/>
+      <c r="B49" s="202"/>
+      <c r="C49" s="210"/>
+      <c r="D49" s="216"/>
     </row>
     <row r="50" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="204"/>
-      <c r="B50" s="205"/>
-      <c r="C50" s="199"/>
-      <c r="D50" s="226"/>
+      <c r="A50" s="203"/>
+      <c r="B50" s="202"/>
+      <c r="C50" s="210"/>
+      <c r="D50" s="217"/>
     </row>
     <row r="51" spans="1:4" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="39" t="s">
@@ -31856,10 +31890,10 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="205" t="s">
+      <c r="A53" s="202" t="s">
         <v>84</v>
       </c>
-      <c r="B53" s="205" t="s">
+      <c r="B53" s="202" t="s">
         <v>185</v>
       </c>
       <c r="C53" s="78" t="s">
@@ -31870,8 +31904,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="205"/>
-      <c r="B54" s="205"/>
+      <c r="A54" s="202"/>
+      <c r="B54" s="202"/>
       <c r="C54" s="78" t="s">
         <v>190</v>
       </c>
@@ -31880,8 +31914,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="205"/>
-      <c r="B55" s="205"/>
+      <c r="A55" s="202"/>
+      <c r="B55" s="202"/>
       <c r="C55" s="78" t="s">
         <v>205</v>
       </c>
@@ -31890,9 +31924,9 @@
       </c>
     </row>
     <row r="56" spans="1:4" ht="34.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="205"/>
-      <c r="B56" s="205"/>
-      <c r="C56" s="230" t="s">
+      <c r="A56" s="202"/>
+      <c r="B56" s="202"/>
+      <c r="C56" s="221" t="s">
         <v>208</v>
       </c>
       <c r="D56" s="79" t="s">
@@ -31900,16 +31934,16 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="205"/>
-      <c r="B57" s="205"/>
-      <c r="C57" s="230"/>
+      <c r="A57" s="202"/>
+      <c r="B57" s="202"/>
+      <c r="C57" s="221"/>
       <c r="D57" s="47" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="205"/>
-      <c r="B58" s="205"/>
+      <c r="A58" s="202"/>
+      <c r="B58" s="202"/>
       <c r="C58" s="78" t="s">
         <v>209</v>
       </c>
@@ -31918,8 +31952,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="205"/>
-      <c r="B59" s="205"/>
+      <c r="A59" s="202"/>
+      <c r="B59" s="202"/>
       <c r="C59" s="78" t="s">
         <v>210</v>
       </c>
@@ -31928,9 +31962,9 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="205"/>
-      <c r="B60" s="205"/>
-      <c r="C60" s="230" t="s">
+      <c r="A60" s="202"/>
+      <c r="B60" s="202"/>
+      <c r="C60" s="221" t="s">
         <v>207</v>
       </c>
       <c r="D60" s="46" t="s">
@@ -31938,25 +31972,25 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="205"/>
-      <c r="B61" s="205"/>
-      <c r="C61" s="230"/>
+      <c r="A61" s="202"/>
+      <c r="B61" s="202"/>
+      <c r="C61" s="221"/>
       <c r="D61" s="46" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="205"/>
-      <c r="B62" s="205"/>
-      <c r="C62" s="230"/>
+      <c r="A62" s="202"/>
+      <c r="B62" s="202"/>
+      <c r="C62" s="221"/>
       <c r="D62" s="79" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="205"/>
-      <c r="B63" s="205"/>
-      <c r="C63" s="223" t="s">
+      <c r="A63" s="202"/>
+      <c r="B63" s="202"/>
+      <c r="C63" s="222" t="s">
         <v>206</v>
       </c>
       <c r="D63" s="45" t="s">
@@ -31964,30 +31998,30 @@
       </c>
     </row>
     <row r="64" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="205"/>
-      <c r="B64" s="205"/>
-      <c r="C64" s="223"/>
-      <c r="D64" s="206" t="s">
+      <c r="A64" s="202"/>
+      <c r="B64" s="202"/>
+      <c r="C64" s="222"/>
+      <c r="D64" s="204" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="12.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="205"/>
-      <c r="B65" s="205"/>
-      <c r="C65" s="223"/>
-      <c r="D65" s="206"/>
+      <c r="A65" s="202"/>
+      <c r="B65" s="202"/>
+      <c r="C65" s="222"/>
+      <c r="D65" s="204"/>
     </row>
     <row r="66" spans="1:4" ht="13.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="205"/>
-      <c r="B66" s="205"/>
-      <c r="C66" s="223"/>
-      <c r="D66" s="206"/>
+      <c r="A66" s="202"/>
+      <c r="B66" s="202"/>
+      <c r="C66" s="222"/>
+      <c r="D66" s="204"/>
     </row>
     <row r="67" spans="1:4" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="205"/>
-      <c r="B67" s="205"/>
-      <c r="C67" s="223"/>
-      <c r="D67" s="206"/>
+      <c r="A67" s="202"/>
+      <c r="B67" s="202"/>
+      <c r="C67" s="222"/>
+      <c r="D67" s="204"/>
     </row>
     <row r="68" spans="1:4" ht="11.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="39"/>
@@ -32043,6 +32077,23 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="A32:A36"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="A4:A9"/>
+    <mergeCell ref="B4:B9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A13:A23"/>
+    <mergeCell ref="B13:B23"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="C13:C23"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C43:C44"/>
     <mergeCell ref="D64:D67"/>
     <mergeCell ref="D41:D42"/>
     <mergeCell ref="D46:D50"/>
@@ -32059,23 +32110,6 @@
     <mergeCell ref="B45:B50"/>
     <mergeCell ref="C49:C50"/>
     <mergeCell ref="C63:C67"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="C13:C23"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="A32:A36"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="A4:A9"/>
-    <mergeCell ref="B4:B9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="A13:A23"/>
-    <mergeCell ref="B13:B23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -32084,7 +32118,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D294"/>
+  <dimension ref="A1:D298"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="62.42578125" customWidth="1"/>
@@ -32116,10 +32150,10 @@
       <c r="D2" s="104"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="255" t="s">
+      <c r="A3" s="232" t="s">
         <v>434</v>
       </c>
-      <c r="B3" s="255" t="s">
+      <c r="B3" s="232" t="s">
         <v>435</v>
       </c>
       <c r="C3" s="101" t="s">
@@ -32130,8 +32164,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="256"/>
-      <c r="B4" s="256"/>
+      <c r="A4" s="233"/>
+      <c r="B4" s="233"/>
       <c r="C4" s="100" t="s">
         <v>438</v>
       </c>
@@ -32140,8 +32174,8 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="257"/>
-      <c r="B5" s="257"/>
+      <c r="A5" s="234"/>
+      <c r="B5" s="234"/>
       <c r="C5" s="100" t="s">
         <v>438</v>
       </c>
@@ -32164,10 +32198,10 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="255" t="s">
+      <c r="A7" s="232" t="s">
         <v>485</v>
       </c>
-      <c r="B7" s="255" t="s">
+      <c r="B7" s="232" t="s">
         <v>435</v>
       </c>
       <c r="C7" s="141" t="s">
@@ -32178,8 +32212,8 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="256"/>
-      <c r="B8" s="256"/>
+      <c r="A8" s="233"/>
+      <c r="B8" s="233"/>
       <c r="C8" s="141" t="s">
         <v>486</v>
       </c>
@@ -32188,8 +32222,8 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="257"/>
-      <c r="B9" s="257"/>
+      <c r="A9" s="234"/>
+      <c r="B9" s="234"/>
       <c r="C9" s="141" t="s">
         <v>489</v>
       </c>
@@ -32206,7 +32240,7 @@
       <c r="D10" s="127"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="243" t="s">
+      <c r="A11" s="240" t="s">
         <v>248</v>
       </c>
       <c r="B11" s="235" t="s">
@@ -32220,8 +32254,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="245"/>
-      <c r="B12" s="236"/>
+      <c r="A12" s="241"/>
+      <c r="B12" s="237"/>
       <c r="C12" s="128" t="s">
         <v>451</v>
       </c>
@@ -32244,7 +32278,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="237"/>
+      <c r="A14" s="236"/>
       <c r="B14" s="151"/>
       <c r="C14" s="106" t="s">
         <v>300</v>
@@ -32254,7 +32288,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="237"/>
+      <c r="A15" s="236"/>
       <c r="B15" s="151"/>
       <c r="C15" s="128" t="s">
         <v>281</v>
@@ -32264,7 +32298,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="237"/>
+      <c r="A16" s="236"/>
       <c r="B16" s="151"/>
       <c r="C16" s="128" t="s">
         <v>21</v>
@@ -32274,7 +32308,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="237"/>
+      <c r="A17" s="236"/>
       <c r="B17" s="150"/>
       <c r="C17" s="128" t="s">
         <v>449</v>
@@ -32284,7 +32318,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="236"/>
+      <c r="A18" s="237"/>
       <c r="B18" s="151"/>
       <c r="C18" s="128" t="s">
         <v>436</v>
@@ -32308,7 +32342,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="243" t="s">
+      <c r="A20" s="240" t="s">
         <v>454</v>
       </c>
       <c r="B20" s="235" t="s">
@@ -32322,8 +32356,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="245"/>
-      <c r="B21" s="236"/>
+      <c r="A21" s="241"/>
+      <c r="B21" s="237"/>
       <c r="C21" s="128"/>
       <c r="D21" s="106" t="s">
         <v>479</v>
@@ -32338,10 +32372,10 @@
       <c r="D22" s="104"/>
     </row>
     <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="260" t="s">
+      <c r="A23" s="242" t="s">
         <v>337</v>
       </c>
-      <c r="B23" s="261" t="s">
+      <c r="B23" s="243" t="s">
         <v>432</v>
       </c>
       <c r="C23" s="100" t="s">
@@ -32352,8 +32386,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="260"/>
-      <c r="B24" s="261"/>
+      <c r="A24" s="242"/>
+      <c r="B24" s="243"/>
       <c r="C24" s="100" t="s">
         <v>342</v>
       </c>
@@ -32362,8 +32396,8 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="260"/>
-      <c r="B25" s="261"/>
+      <c r="A25" s="242"/>
+      <c r="B25" s="243"/>
       <c r="C25" s="100" t="s">
         <v>338</v>
       </c>
@@ -32380,7 +32414,7 @@
       <c r="D26" s="104"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="243" t="s">
+      <c r="A27" s="240" t="s">
         <v>3</v>
       </c>
       <c r="B27" s="235" t="s">
@@ -32392,8 +32426,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="244"/>
-      <c r="B28" s="237"/>
+      <c r="A28" s="246"/>
+      <c r="B28" s="236"/>
       <c r="C28" s="70" t="s">
         <v>234</v>
       </c>
@@ -32402,8 +32436,8 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="244"/>
-      <c r="B29" s="237"/>
+      <c r="A29" s="246"/>
+      <c r="B29" s="236"/>
       <c r="C29" s="140" t="s">
         <v>445</v>
       </c>
@@ -32412,8 +32446,8 @@
       </c>
     </row>
     <row r="30" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="244"/>
-      <c r="B30" s="237"/>
+      <c r="A30" s="246"/>
+      <c r="B30" s="236"/>
       <c r="C30" s="139" t="s">
         <v>480</v>
       </c>
@@ -32422,8 +32456,8 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="244"/>
-      <c r="B31" s="237"/>
+      <c r="A31" s="246"/>
+      <c r="B31" s="236"/>
       <c r="C31" s="147" t="s">
         <v>491</v>
       </c>
@@ -32432,8 +32466,8 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="244"/>
-      <c r="B32" s="237"/>
+      <c r="A32" s="246"/>
+      <c r="B32" s="236"/>
       <c r="C32" s="147" t="s">
         <v>480</v>
       </c>
@@ -32442,7 +32476,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="243" t="s">
+      <c r="A33" s="240" t="s">
         <v>74</v>
       </c>
       <c r="B33" s="235" t="s">
@@ -32456,8 +32490,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="244"/>
-      <c r="B34" s="237"/>
+      <c r="A34" s="246"/>
+      <c r="B34" s="236"/>
       <c r="C34" s="131" t="s">
         <v>467</v>
       </c>
@@ -32466,8 +32500,8 @@
       </c>
     </row>
     <row r="35" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="245"/>
-      <c r="B35" s="236"/>
+      <c r="A35" s="241"/>
+      <c r="B35" s="237"/>
       <c r="C35" s="136" t="s">
         <v>457</v>
       </c>
@@ -32516,10 +32550,10 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="251" t="s">
+      <c r="A39" s="245" t="s">
         <v>270</v>
       </c>
-      <c r="B39" s="252" t="s">
+      <c r="B39" s="244" t="s">
         <v>432</v>
       </c>
       <c r="C39" s="106"/>
@@ -32528,8 +32562,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="251"/>
-      <c r="B40" s="252"/>
+      <c r="A40" s="245"/>
+      <c r="B40" s="244"/>
       <c r="C40" s="106" t="s">
         <v>494</v>
       </c>
@@ -32538,16 +32572,16 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="251"/>
-      <c r="B41" s="252"/>
+      <c r="A41" s="245"/>
+      <c r="B41" s="244"/>
       <c r="C41" s="106"/>
       <c r="D41" s="106" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="251"/>
-      <c r="B42" s="252"/>
+      <c r="A42" s="245"/>
+      <c r="B42" s="244"/>
       <c r="C42" s="110" t="s">
         <v>320</v>
       </c>
@@ -32556,8 +32590,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="251"/>
-      <c r="B43" s="252"/>
+      <c r="A43" s="245"/>
+      <c r="B43" s="244"/>
       <c r="C43" s="111" t="s">
         <v>399</v>
       </c>
@@ -32578,7 +32612,7 @@
       <c r="D44" s="106"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="258" t="s">
+      <c r="A45" s="238" t="s">
         <v>165</v>
       </c>
       <c r="B45" s="235" t="s">
@@ -32590,8 +32624,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="259"/>
-      <c r="B46" s="237"/>
+      <c r="A46" s="239"/>
+      <c r="B46" s="236"/>
       <c r="C46" s="111" t="s">
         <v>356</v>
       </c>
@@ -32600,8 +32634,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="259"/>
-      <c r="B47" s="237"/>
+      <c r="A47" s="239"/>
+      <c r="B47" s="236"/>
       <c r="C47" s="111" t="s">
         <v>354</v>
       </c>
@@ -32610,8 +32644,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="259"/>
-      <c r="B48" s="237"/>
+      <c r="A48" s="239"/>
+      <c r="B48" s="236"/>
       <c r="C48" s="114" t="s">
         <v>362</v>
       </c>
@@ -32620,8 +32654,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="259"/>
-      <c r="B49" s="237"/>
+      <c r="A49" s="239"/>
+      <c r="B49" s="236"/>
       <c r="C49" s="111" t="s">
         <v>354</v>
       </c>
@@ -32630,8 +32664,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="259"/>
-      <c r="B50" s="237"/>
+      <c r="A50" s="239"/>
+      <c r="B50" s="236"/>
       <c r="C50" s="111" t="s">
         <v>366</v>
       </c>
@@ -32640,8 +32674,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="259"/>
-      <c r="B51" s="237"/>
+      <c r="A51" s="239"/>
+      <c r="B51" s="236"/>
       <c r="C51" s="111" t="s">
         <v>354</v>
       </c>
@@ -32650,8 +32684,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="259"/>
-      <c r="B52" s="237"/>
+      <c r="A52" s="239"/>
+      <c r="B52" s="236"/>
       <c r="C52" s="130" t="s">
         <v>461</v>
       </c>
@@ -32660,8 +32694,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="259"/>
-      <c r="B53" s="237"/>
+      <c r="A53" s="239"/>
+      <c r="B53" s="236"/>
       <c r="C53" s="130" t="s">
         <v>456</v>
       </c>
@@ -32670,8 +32704,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="259"/>
-      <c r="B54" s="237"/>
+      <c r="A54" s="239"/>
+      <c r="B54" s="236"/>
       <c r="C54" s="130" t="s">
         <v>354</v>
       </c>
@@ -32680,8 +32714,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="259"/>
-      <c r="B55" s="237"/>
+      <c r="A55" s="239"/>
+      <c r="B55" s="236"/>
       <c r="C55" s="130" t="s">
         <v>456</v>
       </c>
@@ -32690,8 +32724,8 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="259"/>
-      <c r="B56" s="237"/>
+      <c r="A56" s="239"/>
+      <c r="B56" s="236"/>
       <c r="C56" s="145" t="s">
         <v>354</v>
       </c>
@@ -32700,8 +32734,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="259"/>
-      <c r="B57" s="237"/>
+      <c r="A57" s="239"/>
+      <c r="B57" s="236"/>
       <c r="C57" s="145" t="s">
         <v>480</v>
       </c>
@@ -32710,8 +32744,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="259"/>
-      <c r="B58" s="237"/>
+      <c r="A58" s="239"/>
+      <c r="B58" s="236"/>
       <c r="C58" s="147" t="s">
         <v>491</v>
       </c>
@@ -32720,8 +32754,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="259"/>
-      <c r="B59" s="237"/>
+      <c r="A59" s="239"/>
+      <c r="B59" s="236"/>
       <c r="C59" s="147" t="s">
         <v>480</v>
       </c>
@@ -32756,7 +32790,7 @@
       <c r="D61" s="112"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="233" t="s">
+      <c r="A62" s="247" t="s">
         <v>364</v>
       </c>
       <c r="B62" s="235" t="s">
@@ -32768,8 +32802,8 @@
       <c r="D62" s="112"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="234"/>
-      <c r="B63" s="236"/>
+      <c r="A63" s="260"/>
+      <c r="B63" s="237"/>
       <c r="C63" s="111" t="s">
         <v>399</v>
       </c>
@@ -32786,7 +32820,7 @@
       <c r="D64" s="103"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="233" t="s">
+      <c r="A65" s="247" t="s">
         <v>236</v>
       </c>
       <c r="B65" s="235" t="s">
@@ -32798,24 +32832,24 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="246"/>
-      <c r="B66" s="237"/>
+      <c r="A66" s="248"/>
+      <c r="B66" s="236"/>
       <c r="C66" s="106"/>
       <c r="D66" s="106" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="246"/>
-      <c r="B67" s="237"/>
+      <c r="A67" s="248"/>
+      <c r="B67" s="236"/>
       <c r="C67" s="106"/>
       <c r="D67" s="106" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="246"/>
-      <c r="B68" s="237"/>
+      <c r="A68" s="248"/>
+      <c r="B68" s="236"/>
       <c r="C68" s="106" t="s">
         <v>295</v>
       </c>
@@ -32824,8 +32858,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="246"/>
-      <c r="B69" s="237"/>
+      <c r="A69" s="248"/>
+      <c r="B69" s="236"/>
       <c r="C69" s="106" t="s">
         <v>323</v>
       </c>
@@ -32834,8 +32868,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="246"/>
-      <c r="B70" s="237"/>
+      <c r="A70" s="248"/>
+      <c r="B70" s="236"/>
       <c r="C70" s="106" t="s">
         <v>368</v>
       </c>
@@ -32844,8 +32878,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="246"/>
-      <c r="B71" s="237"/>
+      <c r="A71" s="248"/>
+      <c r="B71" s="236"/>
       <c r="C71" s="61" t="s">
         <v>472</v>
       </c>
@@ -32854,8 +32888,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="246"/>
-      <c r="B72" s="237"/>
+      <c r="A72" s="248"/>
+      <c r="B72" s="236"/>
       <c r="C72" s="58" t="s">
         <v>37</v>
       </c>
@@ -32864,8 +32898,8 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="246"/>
-      <c r="B73" s="237"/>
+      <c r="A73" s="248"/>
+      <c r="B73" s="236"/>
       <c r="C73" s="137" t="s">
         <v>354</v>
       </c>
@@ -32874,8 +32908,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="246"/>
-      <c r="B74" s="237"/>
+      <c r="A74" s="248"/>
+      <c r="B74" s="236"/>
       <c r="C74" s="137" t="s">
         <v>456</v>
       </c>
@@ -32884,8 +32918,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="246"/>
-      <c r="B75" s="237"/>
+      <c r="A75" s="248"/>
+      <c r="B75" s="236"/>
       <c r="C75" s="137" t="s">
         <v>480</v>
       </c>
@@ -32894,8 +32928,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="246"/>
-      <c r="B76" s="237"/>
+      <c r="A76" s="248"/>
+      <c r="B76" s="236"/>
       <c r="C76" s="146" t="s">
         <v>491</v>
       </c>
@@ -32904,8 +32938,8 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="246"/>
-      <c r="B77" s="237"/>
+      <c r="A77" s="248"/>
+      <c r="B77" s="236"/>
       <c r="C77" s="146" t="s">
         <v>480</v>
       </c>
@@ -32914,7 +32948,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="247" t="s">
+      <c r="A78" s="250" t="s">
         <v>27</v>
       </c>
       <c r="B78" s="235" t="s">
@@ -32928,16 +32962,16 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="248"/>
-      <c r="B79" s="237"/>
+      <c r="A79" s="251"/>
+      <c r="B79" s="236"/>
       <c r="C79" s="106"/>
       <c r="D79" s="106" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A80" s="248"/>
-      <c r="B80" s="237"/>
+      <c r="A80" s="251"/>
+      <c r="B80" s="236"/>
       <c r="C80" s="116" t="s">
         <v>324</v>
       </c>
@@ -32946,8 +32980,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="248"/>
-      <c r="B81" s="237"/>
+      <c r="A81" s="251"/>
+      <c r="B81" s="236"/>
       <c r="C81" s="116" t="s">
         <v>494</v>
       </c>
@@ -32956,8 +32990,8 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="248"/>
-      <c r="B82" s="237"/>
+      <c r="A82" s="251"/>
+      <c r="B82" s="236"/>
       <c r="C82" s="116" t="s">
         <v>354</v>
       </c>
@@ -32966,8 +33000,8 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="248"/>
-      <c r="B83" s="237"/>
+      <c r="A83" s="251"/>
+      <c r="B83" s="236"/>
       <c r="C83" s="116" t="s">
         <v>362</v>
       </c>
@@ -32976,8 +33010,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="248"/>
-      <c r="B84" s="237"/>
+      <c r="A84" s="251"/>
+      <c r="B84" s="236"/>
       <c r="C84" s="116" t="s">
         <v>366</v>
       </c>
@@ -32986,8 +33020,8 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="248"/>
-      <c r="B85" s="237"/>
+      <c r="A85" s="251"/>
+      <c r="B85" s="236"/>
       <c r="C85" s="116" t="s">
         <v>376</v>
       </c>
@@ -32996,8 +33030,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="248"/>
-      <c r="B86" s="237"/>
+      <c r="A86" s="251"/>
+      <c r="B86" s="236"/>
       <c r="C86" s="108" t="s">
         <v>354</v>
       </c>
@@ -33006,8 +33040,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="248"/>
-      <c r="B87" s="237"/>
+      <c r="A87" s="251"/>
+      <c r="B87" s="236"/>
       <c r="C87" s="137" t="s">
         <v>461</v>
       </c>
@@ -33016,8 +33050,8 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="248"/>
-      <c r="B88" s="237"/>
+      <c r="A88" s="251"/>
+      <c r="B88" s="236"/>
       <c r="C88" s="137" t="s">
         <v>456</v>
       </c>
@@ -33026,8 +33060,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="248"/>
-      <c r="B89" s="237"/>
+      <c r="A89" s="251"/>
+      <c r="B89" s="236"/>
       <c r="C89" s="137" t="s">
         <v>354</v>
       </c>
@@ -33036,8 +33070,8 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="248"/>
-      <c r="B90" s="237"/>
+      <c r="A90" s="251"/>
+      <c r="B90" s="236"/>
       <c r="C90" s="137" t="s">
         <v>456</v>
       </c>
@@ -33046,8 +33080,8 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="248"/>
-      <c r="B91" s="237"/>
+      <c r="A91" s="251"/>
+      <c r="B91" s="236"/>
       <c r="C91" s="137" t="s">
         <v>368</v>
       </c>
@@ -33056,8 +33090,8 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="248"/>
-      <c r="B92" s="237"/>
+      <c r="A92" s="251"/>
+      <c r="B92" s="236"/>
       <c r="C92" s="137" t="s">
         <v>354</v>
       </c>
@@ -33066,8 +33100,8 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="248"/>
-      <c r="B93" s="237"/>
+      <c r="A93" s="251"/>
+      <c r="B93" s="236"/>
       <c r="C93" s="137" t="s">
         <v>480</v>
       </c>
@@ -33076,8 +33110,8 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="248"/>
-      <c r="B94" s="237"/>
+      <c r="A94" s="251"/>
+      <c r="B94" s="236"/>
       <c r="C94" s="146" t="s">
         <v>491</v>
       </c>
@@ -33086,8 +33120,8 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="249"/>
-      <c r="B95" s="236"/>
+      <c r="A95" s="252"/>
+      <c r="B95" s="237"/>
       <c r="C95" s="146" t="s">
         <v>480</v>
       </c>
@@ -33096,7 +33130,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="243" t="s">
+      <c r="A96" s="240" t="s">
         <v>222</v>
       </c>
       <c r="B96" s="235" t="s">
@@ -33110,17 +33144,17 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="244"/>
-      <c r="B97" s="237"/>
+      <c r="A97" s="246"/>
+      <c r="B97" s="236"/>
       <c r="C97" s="254"/>
       <c r="D97" s="112" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="244"/>
-      <c r="B98" s="237"/>
-      <c r="C98" s="250" t="s">
+      <c r="A98" s="246"/>
+      <c r="B98" s="236"/>
+      <c r="C98" s="249" t="s">
         <v>239</v>
       </c>
       <c r="D98" s="106" t="s">
@@ -33128,16 +33162,16 @@
       </c>
     </row>
     <row r="99" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A99" s="244"/>
-      <c r="B99" s="237"/>
-      <c r="C99" s="250"/>
+      <c r="A99" s="246"/>
+      <c r="B99" s="236"/>
+      <c r="C99" s="249"/>
       <c r="D99" s="118" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="244"/>
-      <c r="B100" s="237"/>
+      <c r="A100" s="246"/>
+      <c r="B100" s="236"/>
       <c r="C100" s="111" t="s">
         <v>302</v>
       </c>
@@ -33146,8 +33180,8 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="244"/>
-      <c r="B101" s="237"/>
+      <c r="A101" s="246"/>
+      <c r="B101" s="236"/>
       <c r="C101" s="111">
         <v>2.1</v>
       </c>
@@ -33156,8 +33190,8 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="244"/>
-      <c r="B102" s="237"/>
+      <c r="A102" s="246"/>
+      <c r="B102" s="236"/>
       <c r="C102" s="111" t="s">
         <v>238</v>
       </c>
@@ -33166,8 +33200,8 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="244"/>
-      <c r="B103" s="237"/>
+      <c r="A103" s="246"/>
+      <c r="B103" s="236"/>
       <c r="C103" s="111" t="s">
         <v>238</v>
       </c>
@@ -33176,8 +33210,8 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="244"/>
-      <c r="B104" s="237"/>
+      <c r="A104" s="246"/>
+      <c r="B104" s="236"/>
       <c r="C104" s="111" t="s">
         <v>238</v>
       </c>
@@ -33186,8 +33220,8 @@
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="244"/>
-      <c r="B105" s="237"/>
+      <c r="A105" s="246"/>
+      <c r="B105" s="236"/>
       <c r="C105" s="119" t="s">
         <v>373</v>
       </c>
@@ -33196,8 +33230,8 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="244"/>
-      <c r="B106" s="237"/>
+      <c r="A106" s="246"/>
+      <c r="B106" s="236"/>
       <c r="C106" s="111">
         <v>2.1</v>
       </c>
@@ -33206,8 +33240,8 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="244"/>
-      <c r="B107" s="237"/>
+      <c r="A107" s="246"/>
+      <c r="B107" s="236"/>
       <c r="C107" s="111" t="s">
         <v>238</v>
       </c>
@@ -33216,8 +33250,8 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="244"/>
-      <c r="B108" s="237"/>
+      <c r="A108" s="246"/>
+      <c r="B108" s="236"/>
       <c r="C108" s="111" t="s">
         <v>238</v>
       </c>
@@ -33226,8 +33260,8 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="244"/>
-      <c r="B109" s="237"/>
+      <c r="A109" s="246"/>
+      <c r="B109" s="236"/>
       <c r="C109" s="111">
         <v>2.1</v>
       </c>
@@ -33236,7 +33270,7 @@
       </c>
     </row>
     <row r="110" spans="1:4" ht="30.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="247" t="s">
+      <c r="A110" s="250" t="s">
         <v>291</v>
       </c>
       <c r="B110" s="235" t="s">
@@ -33250,8 +33284,8 @@
       </c>
     </row>
     <row r="111" spans="1:4" ht="30.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="248"/>
-      <c r="B111" s="237"/>
+      <c r="A111" s="251"/>
+      <c r="B111" s="236"/>
       <c r="C111" s="106" t="s">
         <v>494</v>
       </c>
@@ -33260,8 +33294,8 @@
       </c>
     </row>
     <row r="112" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A112" s="248"/>
-      <c r="B112" s="237"/>
+      <c r="A112" s="251"/>
+      <c r="B112" s="236"/>
       <c r="C112" s="118" t="s">
         <v>276</v>
       </c>
@@ -33270,8 +33304,8 @@
       </c>
     </row>
     <row r="113" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="249"/>
-      <c r="B113" s="236"/>
+      <c r="A113" s="252"/>
+      <c r="B113" s="237"/>
       <c r="C113" s="106" t="s">
         <v>345</v>
       </c>
@@ -33280,7 +33314,7 @@
       </c>
     </row>
     <row r="114" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="233" t="s">
+      <c r="A114" s="247" t="s">
         <v>365</v>
       </c>
       <c r="B114" s="235" t="s">
@@ -33292,8 +33326,8 @@
       <c r="D114" s="106"/>
     </row>
     <row r="115" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="246"/>
-      <c r="B115" s="237"/>
+      <c r="A115" s="248"/>
+      <c r="B115" s="236"/>
       <c r="C115" s="111" t="s">
         <v>373</v>
       </c>
@@ -33302,8 +33336,8 @@
       </c>
     </row>
     <row r="116" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="246"/>
-      <c r="B116" s="237"/>
+      <c r="A116" s="248"/>
+      <c r="B116" s="236"/>
       <c r="C116" s="111">
         <v>2.1</v>
       </c>
@@ -33312,8 +33346,8 @@
       </c>
     </row>
     <row r="117" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="246"/>
-      <c r="B117" s="237"/>
+      <c r="A117" s="248"/>
+      <c r="B117" s="236"/>
       <c r="C117" s="111" t="s">
         <v>239</v>
       </c>
@@ -33322,8 +33356,8 @@
       </c>
     </row>
     <row r="118" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="246"/>
-      <c r="B118" s="237"/>
+      <c r="A118" s="248"/>
+      <c r="B118" s="236"/>
       <c r="C118" s="111" t="s">
         <v>238</v>
       </c>
@@ -33352,7 +33386,7 @@
       <c r="D120" s="112"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" s="243" t="s">
+      <c r="A121" s="240" t="s">
         <v>256</v>
       </c>
       <c r="B121" s="235" t="s">
@@ -33364,24 +33398,24 @@
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" s="244"/>
-      <c r="B122" s="237"/>
+      <c r="A122" s="246"/>
+      <c r="B122" s="236"/>
       <c r="C122" s="106"/>
       <c r="D122" s="106" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" s="244"/>
-      <c r="B123" s="237"/>
+      <c r="A123" s="246"/>
+      <c r="B123" s="236"/>
       <c r="C123" s="106"/>
       <c r="D123" s="112" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A124" s="244"/>
-      <c r="B124" s="237"/>
+      <c r="A124" s="246"/>
+      <c r="B124" s="236"/>
       <c r="C124" s="106" t="s">
         <v>419</v>
       </c>
@@ -33390,8 +33424,8 @@
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" s="244"/>
-      <c r="B125" s="237"/>
+      <c r="A125" s="246"/>
+      <c r="B125" s="236"/>
       <c r="C125" s="106" t="s">
         <v>424</v>
       </c>
@@ -33400,8 +33434,8 @@
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" s="244"/>
-      <c r="B126" s="237"/>
+      <c r="A126" s="246"/>
+      <c r="B126" s="236"/>
       <c r="C126" s="58" t="s">
         <v>474</v>
       </c>
@@ -33410,8 +33444,8 @@
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A127" s="244"/>
-      <c r="B127" s="237"/>
+      <c r="A127" s="246"/>
+      <c r="B127" s="236"/>
       <c r="C127" s="58" t="s">
         <v>480</v>
       </c>
@@ -33420,10 +33454,10 @@
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="251" t="s">
+      <c r="A128" s="245" t="s">
         <v>329</v>
       </c>
-      <c r="B128" s="252" t="s">
+      <c r="B128" s="244" t="s">
         <v>432</v>
       </c>
       <c r="C128" s="80" t="s">
@@ -33434,8 +33468,8 @@
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A129" s="251"/>
-      <c r="B129" s="252"/>
+      <c r="A129" s="245"/>
+      <c r="B129" s="244"/>
       <c r="C129" s="106" t="s">
         <v>406</v>
       </c>
@@ -33444,42 +33478,42 @@
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A130" s="251"/>
-      <c r="B130" s="252"/>
+      <c r="A130" s="245"/>
+      <c r="B130" s="244"/>
       <c r="C130" s="121" t="s">
         <v>409</v>
       </c>
-      <c r="D130" s="233" t="s">
+      <c r="D130" s="247" t="s">
         <v>413</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A131" s="251"/>
-      <c r="B131" s="252"/>
+      <c r="A131" s="245"/>
+      <c r="B131" s="244"/>
       <c r="C131" s="121" t="s">
         <v>410</v>
       </c>
-      <c r="D131" s="246"/>
+      <c r="D131" s="248"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A132" s="251"/>
-      <c r="B132" s="252"/>
+      <c r="A132" s="245"/>
+      <c r="B132" s="244"/>
       <c r="C132" s="121" t="s">
         <v>411</v>
       </c>
-      <c r="D132" s="246"/>
+      <c r="D132" s="248"/>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A133" s="251"/>
-      <c r="B133" s="252"/>
+      <c r="A133" s="245"/>
+      <c r="B133" s="244"/>
       <c r="C133" s="121" t="s">
         <v>412</v>
       </c>
-      <c r="D133" s="246"/>
+      <c r="D133" s="248"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A134" s="251"/>
-      <c r="B134" s="252"/>
+      <c r="A134" s="245"/>
+      <c r="B134" s="244"/>
       <c r="C134" s="138" t="s">
         <v>475</v>
       </c>
@@ -33502,7 +33536,7 @@
       </c>
     </row>
     <row r="136" spans="1:4" ht="30.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="238" t="s">
+      <c r="A136" s="255" t="s">
         <v>32</v>
       </c>
       <c r="B136" s="235" t="s">
@@ -33516,8 +33550,8 @@
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A137" s="239"/>
-      <c r="B137" s="237"/>
+      <c r="A137" s="256"/>
+      <c r="B137" s="236"/>
       <c r="C137" s="106" t="s">
         <v>265</v>
       </c>
@@ -33526,8 +33560,8 @@
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A138" s="239"/>
-      <c r="B138" s="237"/>
+      <c r="A138" s="256"/>
+      <c r="B138" s="236"/>
       <c r="C138" s="106" t="s">
         <v>264</v>
       </c>
@@ -33536,8 +33570,8 @@
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A139" s="239"/>
-      <c r="B139" s="237"/>
+      <c r="A139" s="256"/>
+      <c r="B139" s="236"/>
       <c r="C139" s="112" t="s">
         <v>272</v>
       </c>
@@ -33546,8 +33580,8 @@
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A140" s="239"/>
-      <c r="B140" s="237"/>
+      <c r="A140" s="256"/>
+      <c r="B140" s="236"/>
       <c r="C140" s="106" t="s">
         <v>277</v>
       </c>
@@ -33556,8 +33590,8 @@
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A141" s="239"/>
-      <c r="B141" s="237"/>
+      <c r="A141" s="256"/>
+      <c r="B141" s="236"/>
       <c r="C141" s="106" t="s">
         <v>278</v>
       </c>
@@ -33566,8 +33600,8 @@
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A142" s="239"/>
-      <c r="B142" s="237"/>
+      <c r="A142" s="256"/>
+      <c r="B142" s="236"/>
       <c r="C142" s="112" t="s">
         <v>283</v>
       </c>
@@ -33576,8 +33610,8 @@
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A143" s="239"/>
-      <c r="B143" s="237"/>
+      <c r="A143" s="256"/>
+      <c r="B143" s="236"/>
       <c r="C143" s="112" t="s">
         <v>297</v>
       </c>
@@ -33586,8 +33620,8 @@
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A144" s="239"/>
-      <c r="B144" s="237"/>
+      <c r="A144" s="256"/>
+      <c r="B144" s="236"/>
       <c r="C144" s="112" t="s">
         <v>284</v>
       </c>
@@ -33596,8 +33630,8 @@
       </c>
     </row>
     <row r="145" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A145" s="239"/>
-      <c r="B145" s="237"/>
+      <c r="A145" s="256"/>
+      <c r="B145" s="236"/>
       <c r="C145" s="122" t="s">
         <v>243</v>
       </c>
@@ -33606,8 +33640,8 @@
       </c>
     </row>
     <row r="146" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A146" s="239"/>
-      <c r="B146" s="237"/>
+      <c r="A146" s="256"/>
+      <c r="B146" s="236"/>
       <c r="C146" s="116" t="s">
         <v>306</v>
       </c>
@@ -33616,8 +33650,8 @@
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A147" s="239"/>
-      <c r="B147" s="237"/>
+      <c r="A147" s="256"/>
+      <c r="B147" s="236"/>
       <c r="C147" s="106" t="s">
         <v>307</v>
       </c>
@@ -33626,8 +33660,8 @@
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A148" s="239"/>
-      <c r="B148" s="237"/>
+      <c r="A148" s="256"/>
+      <c r="B148" s="236"/>
       <c r="C148" s="112" t="s">
         <v>308</v>
       </c>
@@ -33636,8 +33670,8 @@
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" s="239"/>
-      <c r="B149" s="237"/>
+      <c r="A149" s="256"/>
+      <c r="B149" s="236"/>
       <c r="C149" s="112" t="s">
         <v>310</v>
       </c>
@@ -33646,8 +33680,8 @@
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A150" s="239"/>
-      <c r="B150" s="237"/>
+      <c r="A150" s="256"/>
+      <c r="B150" s="236"/>
       <c r="C150" s="112" t="s">
         <v>263</v>
       </c>
@@ -33656,8 +33690,8 @@
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A151" s="239"/>
-      <c r="B151" s="237"/>
+      <c r="A151" s="256"/>
+      <c r="B151" s="236"/>
       <c r="C151" s="106" t="s">
         <v>313</v>
       </c>
@@ -33666,8 +33700,8 @@
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A152" s="239"/>
-      <c r="B152" s="237"/>
+      <c r="A152" s="256"/>
+      <c r="B152" s="236"/>
       <c r="C152" s="112" t="s">
         <v>278</v>
       </c>
@@ -33676,8 +33710,8 @@
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A153" s="239"/>
-      <c r="B153" s="237"/>
+      <c r="A153" s="256"/>
+      <c r="B153" s="236"/>
       <c r="C153" s="112" t="s">
         <v>314</v>
       </c>
@@ -33686,16 +33720,16 @@
       </c>
     </row>
     <row r="154" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A154" s="239"/>
-      <c r="B154" s="237"/>
+      <c r="A154" s="256"/>
+      <c r="B154" s="236"/>
       <c r="C154" s="106"/>
       <c r="D154" s="97" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A155" s="239"/>
-      <c r="B155" s="237"/>
+      <c r="A155" s="256"/>
+      <c r="B155" s="236"/>
       <c r="C155" s="112" t="s">
         <v>317</v>
       </c>
@@ -33704,8 +33738,8 @@
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A156" s="239"/>
-      <c r="B156" s="237"/>
+      <c r="A156" s="256"/>
+      <c r="B156" s="236"/>
       <c r="C156" s="112" t="s">
         <v>263</v>
       </c>
@@ -33714,8 +33748,8 @@
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A157" s="239"/>
-      <c r="B157" s="237"/>
+      <c r="A157" s="256"/>
+      <c r="B157" s="236"/>
       <c r="C157" s="112" t="s">
         <v>334</v>
       </c>
@@ -33724,8 +33758,8 @@
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A158" s="239"/>
-      <c r="B158" s="237"/>
+      <c r="A158" s="256"/>
+      <c r="B158" s="236"/>
       <c r="C158" s="112" t="s">
         <v>335</v>
       </c>
@@ -33734,8 +33768,8 @@
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A159" s="239"/>
-      <c r="B159" s="237"/>
+      <c r="A159" s="256"/>
+      <c r="B159" s="236"/>
       <c r="C159" s="112" t="s">
         <v>319</v>
       </c>
@@ -33744,8 +33778,8 @@
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A160" s="239"/>
-      <c r="B160" s="237"/>
+      <c r="A160" s="256"/>
+      <c r="B160" s="236"/>
       <c r="C160" s="117" t="s">
         <v>340</v>
       </c>
@@ -33754,8 +33788,8 @@
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A161" s="239"/>
-      <c r="B161" s="237"/>
+      <c r="A161" s="256"/>
+      <c r="B161" s="236"/>
       <c r="C161" s="112" t="s">
         <v>333</v>
       </c>
@@ -33764,8 +33798,8 @@
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A162" s="239"/>
-      <c r="B162" s="237"/>
+      <c r="A162" s="256"/>
+      <c r="B162" s="236"/>
       <c r="C162" s="112" t="s">
         <v>348</v>
       </c>
@@ -33774,8 +33808,8 @@
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A163" s="239"/>
-      <c r="B163" s="237"/>
+      <c r="A163" s="256"/>
+      <c r="B163" s="236"/>
       <c r="C163" s="101" t="s">
         <v>351</v>
       </c>
@@ -33784,8 +33818,8 @@
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A164" s="239"/>
-      <c r="B164" s="237"/>
+      <c r="A164" s="256"/>
+      <c r="B164" s="236"/>
       <c r="C164" s="112" t="s">
         <v>352</v>
       </c>
@@ -33794,8 +33828,8 @@
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A165" s="239"/>
-      <c r="B165" s="237"/>
+      <c r="A165" s="256"/>
+      <c r="B165" s="236"/>
       <c r="C165" s="112" t="s">
         <v>353</v>
       </c>
@@ -33804,8 +33838,8 @@
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A166" s="239"/>
-      <c r="B166" s="237"/>
+      <c r="A166" s="256"/>
+      <c r="B166" s="236"/>
       <c r="C166" s="112" t="s">
         <v>359</v>
       </c>
@@ -33814,8 +33848,8 @@
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A167" s="239"/>
-      <c r="B167" s="237"/>
+      <c r="A167" s="256"/>
+      <c r="B167" s="236"/>
       <c r="C167" s="112" t="s">
         <v>361</v>
       </c>
@@ -33824,8 +33858,8 @@
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A168" s="239"/>
-      <c r="B168" s="237"/>
+      <c r="A168" s="256"/>
+      <c r="B168" s="236"/>
       <c r="C168" s="112" t="s">
         <v>367</v>
       </c>
@@ -33834,8 +33868,8 @@
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A169" s="239"/>
-      <c r="B169" s="237"/>
+      <c r="A169" s="256"/>
+      <c r="B169" s="236"/>
       <c r="C169" s="112" t="s">
         <v>359</v>
       </c>
@@ -33844,8 +33878,8 @@
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A170" s="239"/>
-      <c r="B170" s="237"/>
+      <c r="A170" s="256"/>
+      <c r="B170" s="236"/>
       <c r="C170" s="117" t="s">
         <v>380</v>
       </c>
@@ -33854,8 +33888,8 @@
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A171" s="239"/>
-      <c r="B171" s="237"/>
+      <c r="A171" s="256"/>
+      <c r="B171" s="236"/>
       <c r="C171" s="106" t="s">
         <v>384</v>
       </c>
@@ -33864,8 +33898,8 @@
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A172" s="239"/>
-      <c r="B172" s="237"/>
+      <c r="A172" s="256"/>
+      <c r="B172" s="236"/>
       <c r="C172" s="106" t="s">
         <v>387</v>
       </c>
@@ -33874,8 +33908,8 @@
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A173" s="239"/>
-      <c r="B173" s="237"/>
+      <c r="A173" s="256"/>
+      <c r="B173" s="236"/>
       <c r="C173" s="106" t="s">
         <v>388</v>
       </c>
@@ -33884,8 +33918,8 @@
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A174" s="239"/>
-      <c r="B174" s="237"/>
+      <c r="A174" s="256"/>
+      <c r="B174" s="236"/>
       <c r="C174" s="106" t="s">
         <v>389</v>
       </c>
@@ -33894,8 +33928,8 @@
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A175" s="239"/>
-      <c r="B175" s="237"/>
+      <c r="A175" s="256"/>
+      <c r="B175" s="236"/>
       <c r="C175" s="106" t="s">
         <v>390</v>
       </c>
@@ -33904,8 +33938,8 @@
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A176" s="239"/>
-      <c r="B176" s="237"/>
+      <c r="A176" s="256"/>
+      <c r="B176" s="236"/>
       <c r="C176" s="106" t="s">
         <v>391</v>
       </c>
@@ -33914,8 +33948,8 @@
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A177" s="239"/>
-      <c r="B177" s="237"/>
+      <c r="A177" s="256"/>
+      <c r="B177" s="236"/>
       <c r="C177" s="106" t="s">
         <v>394</v>
       </c>
@@ -33924,8 +33958,8 @@
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A178" s="239"/>
-      <c r="B178" s="237"/>
+      <c r="A178" s="256"/>
+      <c r="B178" s="236"/>
       <c r="C178" s="106" t="s">
         <v>404</v>
       </c>
@@ -33934,8 +33968,8 @@
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A179" s="239"/>
-      <c r="B179" s="237"/>
+      <c r="A179" s="256"/>
+      <c r="B179" s="236"/>
       <c r="C179" s="106" t="s">
         <v>405</v>
       </c>
@@ -33944,8 +33978,8 @@
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A180" s="239"/>
-      <c r="B180" s="237"/>
+      <c r="A180" s="256"/>
+      <c r="B180" s="236"/>
       <c r="C180" s="106" t="s">
         <v>422</v>
       </c>
@@ -33954,8 +33988,8 @@
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A181" s="239"/>
-      <c r="B181" s="237"/>
+      <c r="A181" s="256"/>
+      <c r="B181" s="236"/>
       <c r="C181" s="106" t="s">
         <v>423</v>
       </c>
@@ -33964,8 +33998,8 @@
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A182" s="239"/>
-      <c r="B182" s="237"/>
+      <c r="A182" s="256"/>
+      <c r="B182" s="236"/>
       <c r="C182" s="106" t="s">
         <v>426</v>
       </c>
@@ -33974,8 +34008,8 @@
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A183" s="239"/>
-      <c r="B183" s="237"/>
+      <c r="A183" s="256"/>
+      <c r="B183" s="236"/>
       <c r="C183" s="58" t="s">
         <v>477</v>
       </c>
@@ -33984,8 +34018,8 @@
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A184" s="239"/>
-      <c r="B184" s="237"/>
+      <c r="A184" s="256"/>
+      <c r="B184" s="236"/>
       <c r="C184" s="106" t="s">
         <v>422</v>
       </c>
@@ -33994,8 +34028,8 @@
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A185" s="239"/>
-      <c r="B185" s="237"/>
+      <c r="A185" s="256"/>
+      <c r="B185" s="236"/>
       <c r="C185" s="106" t="s">
         <v>476</v>
       </c>
@@ -34004,8 +34038,8 @@
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A186" s="240"/>
-      <c r="B186" s="236"/>
+      <c r="A186" s="257"/>
+      <c r="B186" s="237"/>
       <c r="C186" s="112" t="s">
         <v>333</v>
       </c>
@@ -34014,7 +34048,7 @@
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A187" s="238" t="s">
+      <c r="A187" s="255" t="s">
         <v>416</v>
       </c>
       <c r="B187" s="235" t="s">
@@ -34028,8 +34062,8 @@
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A188" s="239"/>
-      <c r="B188" s="237"/>
+      <c r="A188" s="256"/>
+      <c r="B188" s="236"/>
       <c r="C188" s="58" t="s">
         <v>478</v>
       </c>
@@ -34038,8 +34072,8 @@
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A189" s="240"/>
-      <c r="B189" s="236"/>
+      <c r="A189" s="257"/>
+      <c r="B189" s="237"/>
       <c r="C189" s="58" t="s">
         <v>483</v>
       </c>
@@ -34084,7 +34118,7 @@
       <c r="D192" s="104"/>
     </row>
     <row r="193" spans="1:4" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A193" s="243" t="s">
+      <c r="A193" s="240" t="s">
         <v>84</v>
       </c>
       <c r="B193" s="235" t="s">
@@ -34096,8 +34130,8 @@
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A194" s="244"/>
-      <c r="B194" s="237"/>
+      <c r="A194" s="246"/>
+      <c r="B194" s="236"/>
       <c r="C194" s="70" t="s">
         <v>245</v>
       </c>
@@ -34106,8 +34140,8 @@
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A195" s="244"/>
-      <c r="B195" s="237"/>
+      <c r="A195" s="246"/>
+      <c r="B195" s="236"/>
       <c r="C195" s="70">
         <v>10.1</v>
       </c>
@@ -34116,8 +34150,8 @@
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A196" s="244"/>
-      <c r="B196" s="237"/>
+      <c r="A196" s="246"/>
+      <c r="B196" s="236"/>
       <c r="C196" s="70">
         <v>10.199999999999999</v>
       </c>
@@ -34126,8 +34160,8 @@
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A197" s="244"/>
-      <c r="B197" s="237"/>
+      <c r="A197" s="246"/>
+      <c r="B197" s="236"/>
       <c r="C197" s="98" t="s">
         <v>288</v>
       </c>
@@ -34136,8 +34170,8 @@
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A198" s="244"/>
-      <c r="B198" s="237"/>
+      <c r="A198" s="246"/>
+      <c r="B198" s="236"/>
       <c r="C198" s="98" t="s">
         <v>370</v>
       </c>
@@ -34146,8 +34180,8 @@
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A199" s="244"/>
-      <c r="B199" s="237"/>
+      <c r="A199" s="246"/>
+      <c r="B199" s="236"/>
       <c r="C199" s="98" t="s">
         <v>117</v>
       </c>
@@ -34156,8 +34190,8 @@
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A200" s="244"/>
-      <c r="B200" s="237"/>
+      <c r="A200" s="246"/>
+      <c r="B200" s="236"/>
       <c r="C200" s="98" t="s">
         <v>417</v>
       </c>
@@ -34166,8 +34200,8 @@
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A201" s="244"/>
-      <c r="B201" s="237"/>
+      <c r="A201" s="246"/>
+      <c r="B201" s="236"/>
       <c r="C201" s="98" t="s">
         <v>17</v>
       </c>
@@ -34176,8 +34210,8 @@
       </c>
     </row>
     <row r="202" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A202" s="245"/>
-      <c r="B202" s="236"/>
+      <c r="A202" s="241"/>
+      <c r="B202" s="237"/>
       <c r="C202" s="98" t="s">
         <v>460</v>
       </c>
@@ -34186,7 +34220,7 @@
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A203" s="243" t="s">
+      <c r="A203" s="240" t="s">
         <v>246</v>
       </c>
       <c r="B203" s="235" t="s">
@@ -34198,8 +34232,8 @@
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A204" s="244"/>
-      <c r="B204" s="237"/>
+      <c r="A204" s="246"/>
+      <c r="B204" s="236"/>
       <c r="C204" s="125" t="s">
         <v>428</v>
       </c>
@@ -34230,7 +34264,7 @@
       <c r="D206" s="127"/>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A207" s="243" t="s">
+      <c r="A207" s="240" t="s">
         <v>58</v>
       </c>
       <c r="B207" s="235" t="s">
@@ -34244,8 +34278,8 @@
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A208" s="244"/>
-      <c r="B208" s="237"/>
+      <c r="A208" s="246"/>
+      <c r="B208" s="236"/>
       <c r="C208" s="128" t="s">
         <v>260</v>
       </c>
@@ -34254,15 +34288,15 @@
       </c>
     </row>
     <row r="209" spans="1:4" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A209" s="245"/>
-      <c r="B209" s="236"/>
+      <c r="A209" s="241"/>
+      <c r="B209" s="237"/>
       <c r="C209" s="106"/>
       <c r="D209" s="106" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A210" s="241" t="s">
+      <c r="A210" s="261" t="s">
         <v>59</v>
       </c>
       <c r="B210" s="235" t="s">
@@ -34276,15 +34310,15 @@
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A211" s="242"/>
-      <c r="B211" s="236"/>
+      <c r="A211" s="262"/>
+      <c r="B211" s="237"/>
       <c r="C211" s="118"/>
       <c r="D211" s="106" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A212" s="241" t="s">
+      <c r="A212" s="261" t="s">
         <v>286</v>
       </c>
       <c r="B212" s="235" t="s">
@@ -34296,15 +34330,15 @@
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A213" s="242"/>
-      <c r="B213" s="236"/>
+      <c r="A213" s="262"/>
+      <c r="B213" s="237"/>
       <c r="C213" s="106"/>
       <c r="D213" s="106" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A214" s="241" t="s">
+      <c r="A214" s="261" t="s">
         <v>60</v>
       </c>
       <c r="B214" s="235" t="s">
@@ -34318,8 +34352,8 @@
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A215" s="242"/>
-      <c r="B215" s="236"/>
+      <c r="A215" s="262"/>
+      <c r="B215" s="237"/>
       <c r="C215" s="106"/>
       <c r="D215" s="106" t="s">
         <v>408</v>
@@ -34922,10 +34956,10 @@
       <c r="D265" s="173"/>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A266" s="196" t="s">
+      <c r="A266" s="201" t="s">
         <v>499</v>
       </c>
-      <c r="B266" s="230" t="s">
+      <c r="B266" s="221" t="s">
         <v>432</v>
       </c>
       <c r="C266" s="168" t="s">
@@ -34936,8 +34970,8 @@
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A267" s="196"/>
-      <c r="B267" s="230"/>
+      <c r="A267" s="201"/>
+      <c r="B267" s="221"/>
       <c r="C267" s="168" t="s">
         <v>535</v>
       </c>
@@ -34960,10 +34994,10 @@
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A269" s="201" t="s">
+      <c r="A269" s="212" t="s">
         <v>540</v>
       </c>
-      <c r="B269" s="231" t="s">
+      <c r="B269" s="258" t="s">
         <v>432</v>
       </c>
       <c r="C269" s="168" t="s">
@@ -34974,8 +35008,8 @@
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A270" s="202"/>
-      <c r="B270" s="232"/>
+      <c r="A270" s="213"/>
+      <c r="B270" s="259"/>
       <c r="C270" s="168" t="s">
         <v>543</v>
       </c>
@@ -35286,7 +35320,7 @@
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A293" s="262" t="s">
+      <c r="A293" s="181" t="s">
         <v>579</v>
       </c>
       <c r="B293" s="180" t="s">
@@ -35313,8 +35347,75 @@
         <v>578</v>
       </c>
     </row>
+    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A295" s="126" t="s">
+        <v>581</v>
+      </c>
+      <c r="B295" s="263"/>
+      <c r="C295" s="264"/>
+      <c r="D295" s="264"/>
+    </row>
+    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A296" s="95" t="s">
+        <v>582</v>
+      </c>
+      <c r="B296" s="266" t="s">
+        <v>583</v>
+      </c>
+      <c r="C296" s="265" t="s">
+        <v>584</v>
+      </c>
+      <c r="D296" s="95" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="298" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B298" s="267"/>
+    </row>
   </sheetData>
   <mergeCells count="58">
+    <mergeCell ref="A269:A270"/>
+    <mergeCell ref="B269:B270"/>
+    <mergeCell ref="A266:A267"/>
+    <mergeCell ref="B266:B267"/>
+    <mergeCell ref="A62:A63"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="B136:B186"/>
+    <mergeCell ref="A136:A186"/>
+    <mergeCell ref="A214:A215"/>
+    <mergeCell ref="B214:B215"/>
+    <mergeCell ref="A210:A211"/>
+    <mergeCell ref="B210:B211"/>
+    <mergeCell ref="A212:A213"/>
+    <mergeCell ref="B212:B213"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="A207:A209"/>
+    <mergeCell ref="B207:B209"/>
+    <mergeCell ref="A193:A202"/>
+    <mergeCell ref="B193:B202"/>
+    <mergeCell ref="A65:A77"/>
+    <mergeCell ref="B65:B77"/>
+    <mergeCell ref="A78:A95"/>
+    <mergeCell ref="B78:B95"/>
+    <mergeCell ref="A203:A204"/>
+    <mergeCell ref="B203:B204"/>
+    <mergeCell ref="B187:B189"/>
+    <mergeCell ref="A187:A189"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="C98:C99"/>
+    <mergeCell ref="A96:A109"/>
+    <mergeCell ref="B96:B109"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="A128:A134"/>
+    <mergeCell ref="B128:B134"/>
+    <mergeCell ref="A114:A118"/>
+    <mergeCell ref="B114:B118"/>
+    <mergeCell ref="A121:A127"/>
+    <mergeCell ref="B121:B127"/>
+    <mergeCell ref="C96:C97"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="A13:A18"/>
@@ -35331,48 +35432,6 @@
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="A27:A32"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="C98:C99"/>
-    <mergeCell ref="A96:A109"/>
-    <mergeCell ref="B96:B109"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="A128:A134"/>
-    <mergeCell ref="B128:B134"/>
-    <mergeCell ref="A114:A118"/>
-    <mergeCell ref="B114:B118"/>
-    <mergeCell ref="A121:A127"/>
-    <mergeCell ref="B121:B127"/>
-    <mergeCell ref="C96:C97"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="A207:A209"/>
-    <mergeCell ref="B207:B209"/>
-    <mergeCell ref="A193:A202"/>
-    <mergeCell ref="B193:B202"/>
-    <mergeCell ref="A65:A77"/>
-    <mergeCell ref="B65:B77"/>
-    <mergeCell ref="A78:A95"/>
-    <mergeCell ref="B78:B95"/>
-    <mergeCell ref="A203:A204"/>
-    <mergeCell ref="B203:B204"/>
-    <mergeCell ref="B187:B189"/>
-    <mergeCell ref="A187:A189"/>
-    <mergeCell ref="A269:A270"/>
-    <mergeCell ref="B269:B270"/>
-    <mergeCell ref="A266:A267"/>
-    <mergeCell ref="B266:B267"/>
-    <mergeCell ref="A62:A63"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="B136:B186"/>
-    <mergeCell ref="A136:A186"/>
-    <mergeCell ref="A214:A215"/>
-    <mergeCell ref="B214:B215"/>
-    <mergeCell ref="A210:A211"/>
-    <mergeCell ref="B210:B211"/>
-    <mergeCell ref="A212:A213"/>
-    <mergeCell ref="B212:B213"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
psr data tems pit3 pit4
</commit_message>
<xml_diff>
--- a/PIT3/Schema Publication Changelog.xlsx
+++ b/PIT3/Schema Publication Changelog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sphilibi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ctrowell\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58FF0AF2-D6B1-4E63-9978-B240AB24CB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AA6EAA-E12C-4619-95BB-7FF0D0ACF732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19080" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-210" yWindow="0" windowWidth="21600" windowHeight="15600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v0.10" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="O'Brien, Ciaran - Personal View" guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="751" activeSheetId="2"/>
+    <customWorkbookView name="Arnold, Eve - Personal View" guid="{057DBB0B-BBF6-4A94-8406-46C99A7DC1D6}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="758" activeSheetId="2"/>
     <customWorkbookView name="Walsh, David P - Personal View" guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1436" windowHeight="675" activeSheetId="2"/>
-    <customWorkbookView name="Arnold, Eve - Personal View" guid="{057DBB0B-BBF6-4A94-8406-46C99A7DC1D6}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="758" activeSheetId="2"/>
-    <customWorkbookView name="O'Brien, Ciaran - Personal View" guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1276" windowHeight="751" activeSheetId="2"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="581">
   <si>
     <t>Document</t>
   </si>
@@ -3625,27 +3625,12 @@
   <si>
     <t>ERR - Enhanced Reporting Submission Request Data Items</t>
   </si>
-  <si>
-    <t>PRSI Exemption Reason Updates</t>
-  </si>
-  <si>
-    <t>Payroll Employer Submission - Employee Level Validation</t>
-  </si>
-  <si>
-    <t>PIT Next Version</t>
-  </si>
-  <si>
-    <t>PRSI Class and Subclass</t>
-  </si>
-  <si>
-    <t>Warning added on PRSI Class and Subclass</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3792,12 +3777,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -4259,7 +4238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="268">
+  <cellXfs count="263">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -4731,9 +4710,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -4779,38 +4755,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -4833,6 +4779,66 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4854,103 +4860,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4962,33 +4890,71 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5354,12 +5320,12 @@
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="182" t="s">
+      <c r="A2" s="181" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="183"/>
-      <c r="C2" s="183"/>
-      <c r="D2" s="184"/>
+      <c r="B2" s="182"/>
+      <c r="C2" s="182"/>
+      <c r="D2" s="183"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -5382,12 +5348,12 @@
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="182" t="s">
+      <c r="A4" s="181" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="183"/>
-      <c r="C4" s="183"/>
-      <c r="D4" s="184"/>
+      <c r="B4" s="182"/>
+      <c r="C4" s="182"/>
+      <c r="D4" s="183"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -5427,10 +5393,10 @@
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="185" t="s">
+      <c r="A7" s="184" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="188">
+      <c r="B7" s="187">
         <v>0.1</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -5444,8 +5410,8 @@
       <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="186"/>
-      <c r="B8" s="189"/>
+      <c r="A8" s="185"/>
+      <c r="B8" s="188"/>
       <c r="C8" s="11" t="s">
         <v>5</v>
       </c>
@@ -5457,8 +5423,8 @@
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="186"/>
-      <c r="B9" s="189"/>
+      <c r="A9" s="185"/>
+      <c r="B9" s="188"/>
       <c r="C9" s="11" t="s">
         <v>6</v>
       </c>
@@ -5470,8 +5436,8 @@
       <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="186"/>
-      <c r="B10" s="189"/>
+      <c r="A10" s="185"/>
+      <c r="B10" s="188"/>
       <c r="C10" s="11" t="s">
         <v>61</v>
       </c>
@@ -5483,8 +5449,8 @@
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="186"/>
-      <c r="B11" s="189"/>
+      <c r="A11" s="185"/>
+      <c r="B11" s="188"/>
       <c r="C11" s="11" t="s">
         <v>73</v>
       </c>
@@ -5496,8 +5462,8 @@
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="187"/>
-      <c r="B12" s="190"/>
+      <c r="A12" s="186"/>
+      <c r="B12" s="189"/>
       <c r="C12" s="11" t="s">
         <v>67</v>
       </c>
@@ -5509,10 +5475,10 @@
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="193" t="s">
+      <c r="A13" s="192" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="188">
+      <c r="B13" s="187">
         <v>0.1</v>
       </c>
       <c r="C13" s="11" t="s">
@@ -5526,8 +5492,8 @@
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="194"/>
-      <c r="B14" s="190"/>
+      <c r="A14" s="193"/>
+      <c r="B14" s="189"/>
       <c r="C14" s="11" t="s">
         <v>69</v>
       </c>
@@ -5573,12 +5539,12 @@
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="182" t="s">
+      <c r="A17" s="181" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="183"/>
-      <c r="C17" s="183"/>
-      <c r="D17" s="184"/>
+      <c r="B17" s="182"/>
+      <c r="C17" s="182"/>
+      <c r="D17" s="183"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -5618,21 +5584,21 @@
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="182" t="s">
+      <c r="A20" s="181" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="183"/>
-      <c r="C20" s="183"/>
-      <c r="D20" s="184"/>
+      <c r="B20" s="182"/>
+      <c r="C20" s="182"/>
+      <c r="D20" s="183"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
     <row r="21" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="195" t="s">
+      <c r="A21" s="194" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="192">
+      <c r="B21" s="191">
         <v>0.1</v>
       </c>
       <c r="C21" s="11" t="s">
@@ -5646,8 +5612,8 @@
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="196"/>
-      <c r="B22" s="190"/>
+      <c r="A22" s="195"/>
+      <c r="B22" s="189"/>
       <c r="C22" s="27" t="s">
         <v>37</v>
       </c>
@@ -5670,18 +5636,18 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="182" t="s">
+      <c r="A24" s="181" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="183"/>
-      <c r="C24" s="183"/>
-      <c r="D24" s="184"/>
+      <c r="B24" s="182"/>
+      <c r="C24" s="182"/>
+      <c r="D24" s="183"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="191" t="s">
+      <c r="A25" s="190" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="192">
+      <c r="B25" s="191">
         <v>0.1</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -5695,8 +5661,8 @@
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="186"/>
-      <c r="B26" s="189"/>
+      <c r="A26" s="185"/>
+      <c r="B26" s="188"/>
       <c r="C26" s="11" t="s">
         <v>71</v>
       </c>
@@ -5708,8 +5674,8 @@
       <c r="G26" s="2"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="186"/>
-      <c r="B27" s="189"/>
+      <c r="A27" s="185"/>
+      <c r="B27" s="188"/>
       <c r="C27" s="11" t="s">
         <v>11</v>
       </c>
@@ -5721,8 +5687,8 @@
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A28" s="186"/>
-      <c r="B28" s="189"/>
+      <c r="A28" s="185"/>
+      <c r="B28" s="188"/>
       <c r="C28" s="21" t="s">
         <v>72</v>
       </c>
@@ -5734,8 +5700,8 @@
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="186"/>
-      <c r="B29" s="189"/>
+      <c r="A29" s="185"/>
+      <c r="B29" s="188"/>
       <c r="C29" s="11" t="s">
         <v>9</v>
       </c>
@@ -5747,8 +5713,8 @@
       <c r="G29" s="2"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="186"/>
-      <c r="B30" s="189"/>
+      <c r="A30" s="185"/>
+      <c r="B30" s="188"/>
       <c r="C30" s="11" t="s">
         <v>13</v>
       </c>
@@ -5760,8 +5726,8 @@
       <c r="G30" s="2"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="186"/>
-      <c r="B31" s="189"/>
+      <c r="A31" s="185"/>
+      <c r="B31" s="188"/>
       <c r="C31" s="11" t="s">
         <v>15</v>
       </c>
@@ -5773,8 +5739,8 @@
       <c r="G31" s="2"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="187"/>
-      <c r="B32" s="190"/>
+      <c r="A32" s="186"/>
+      <c r="B32" s="189"/>
       <c r="C32" s="11" t="s">
         <v>17</v>
       </c>
@@ -5898,12 +5864,12 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="182" t="s">
+      <c r="A41" s="181" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="183"/>
-      <c r="C41" s="183"/>
-      <c r="D41" s="184"/>
+      <c r="B41" s="182"/>
+      <c r="C41" s="182"/>
+      <c r="D41" s="183"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
@@ -5963,7 +5929,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}" topLeftCell="B1">
+    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="B1">
       <selection activeCell="C15" sqref="C15:D15"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5973,7 +5939,7 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
     </customSheetView>
-    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="B1">
+    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}" topLeftCell="B1">
       <selection activeCell="C15" sqref="C15:D15"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
@@ -6078,10 +6044,10 @@
       <c r="D6" s="44"/>
     </row>
     <row r="7" spans="1:4" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="197" t="s">
+      <c r="A7" s="211" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="198" t="s">
+      <c r="B7" s="210" t="s">
         <v>85</v>
       </c>
       <c r="C7" s="43" t="s">
@@ -6092,8 +6058,8 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="197"/>
-      <c r="B8" s="198"/>
+      <c r="A8" s="211"/>
+      <c r="B8" s="210"/>
       <c r="C8" s="38" t="s">
         <v>88</v>
       </c>
@@ -6102,8 +6068,8 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="197"/>
-      <c r="B9" s="198"/>
+      <c r="A9" s="211"/>
+      <c r="B9" s="210"/>
       <c r="C9" s="38" t="s">
         <v>89</v>
       </c>
@@ -6112,8 +6078,8 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="197"/>
-      <c r="B10" s="198"/>
+      <c r="A10" s="211"/>
+      <c r="B10" s="210"/>
       <c r="C10" s="38" t="s">
         <v>6</v>
       </c>
@@ -6122,8 +6088,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="197"/>
-      <c r="B11" s="198"/>
+      <c r="A11" s="211"/>
+      <c r="B11" s="210"/>
       <c r="C11" s="38" t="s">
         <v>93</v>
       </c>
@@ -6132,8 +6098,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="197"/>
-      <c r="B12" s="198"/>
+      <c r="A12" s="211"/>
+      <c r="B12" s="210"/>
       <c r="C12" s="38" t="s">
         <v>96</v>
       </c>
@@ -6142,10 +6108,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="200" t="s">
+      <c r="A13" s="213" t="s">
         <v>146</v>
       </c>
-      <c r="B13" s="198" t="s">
+      <c r="B13" s="210" t="s">
         <v>85</v>
       </c>
       <c r="C13" s="38" t="s">
@@ -6156,8 +6122,8 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="200"/>
-      <c r="B14" s="198"/>
+      <c r="A14" s="213"/>
+      <c r="B14" s="210"/>
       <c r="C14" s="38" t="s">
         <v>180</v>
       </c>
@@ -6166,8 +6132,8 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="200"/>
-      <c r="B15" s="198"/>
+      <c r="A15" s="213"/>
+      <c r="B15" s="210"/>
       <c r="C15" s="43" t="s">
         <v>182</v>
       </c>
@@ -6176,10 +6142,10 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="201" t="s">
+      <c r="A16" s="196" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="202" t="s">
+      <c r="B16" s="205" t="s">
         <v>85</v>
       </c>
       <c r="C16" s="59" t="s">
@@ -6190,8 +6156,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="201"/>
-      <c r="B17" s="202"/>
+      <c r="A17" s="196"/>
+      <c r="B17" s="205"/>
       <c r="C17" s="58" t="s">
         <v>148</v>
       </c>
@@ -6200,8 +6166,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="201"/>
-      <c r="B18" s="202"/>
+      <c r="A18" s="196"/>
+      <c r="B18" s="205"/>
       <c r="C18" s="58" t="s">
         <v>93</v>
       </c>
@@ -6210,8 +6176,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="201"/>
-      <c r="B19" s="202"/>
+      <c r="A19" s="196"/>
+      <c r="B19" s="205"/>
       <c r="C19" s="58" t="s">
         <v>151</v>
       </c>
@@ -6220,8 +6186,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="201"/>
-      <c r="B20" s="202"/>
+      <c r="A20" s="196"/>
+      <c r="B20" s="205"/>
       <c r="C20" s="58" t="s">
         <v>153</v>
       </c>
@@ -6230,8 +6196,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="201"/>
-      <c r="B21" s="202"/>
+      <c r="A21" s="196"/>
+      <c r="B21" s="205"/>
       <c r="C21" s="58" t="s">
         <v>155</v>
       </c>
@@ -6240,8 +6206,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="201"/>
-      <c r="B22" s="202"/>
+      <c r="A22" s="196"/>
+      <c r="B22" s="205"/>
       <c r="C22" s="58" t="s">
         <v>157</v>
       </c>
@@ -6250,8 +6216,8 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="201"/>
-      <c r="B23" s="202"/>
+      <c r="A23" s="196"/>
+      <c r="B23" s="205"/>
       <c r="C23" s="66" t="s">
         <v>159</v>
       </c>
@@ -6260,26 +6226,26 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="201"/>
-      <c r="B24" s="202"/>
-      <c r="C24" s="201" t="s">
+      <c r="A24" s="196"/>
+      <c r="B24" s="205"/>
+      <c r="C24" s="196" t="s">
         <v>161</v>
       </c>
-      <c r="D24" s="208" t="s">
+      <c r="D24" s="197" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="201"/>
-      <c r="B25" s="202"/>
-      <c r="C25" s="201"/>
-      <c r="D25" s="208"/>
+      <c r="A25" s="196"/>
+      <c r="B25" s="205"/>
+      <c r="C25" s="196"/>
+      <c r="D25" s="197"/>
     </row>
     <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="197" t="s">
+      <c r="A26" s="211" t="s">
         <v>163</v>
       </c>
-      <c r="B26" s="198" t="s">
+      <c r="B26" s="210" t="s">
         <v>85</v>
       </c>
       <c r="C26" s="38" t="s">
@@ -6290,8 +6256,8 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="197"/>
-      <c r="B27" s="198"/>
+      <c r="A27" s="211"/>
+      <c r="B27" s="210"/>
       <c r="C27" s="38"/>
       <c r="D27" s="41" t="s">
         <v>118</v>
@@ -6318,28 +6284,28 @@
       <c r="D29" s="39"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="199" t="s">
+      <c r="A30" s="212" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="198" t="s">
+      <c r="B30" s="210" t="s">
         <v>85</v>
       </c>
-      <c r="C30" s="201" t="s">
+      <c r="C30" s="196" t="s">
         <v>169</v>
       </c>
-      <c r="D30" s="211" t="s">
+      <c r="D30" s="200" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="199"/>
-      <c r="B31" s="198"/>
-      <c r="C31" s="201"/>
-      <c r="D31" s="211"/>
+      <c r="A31" s="212"/>
+      <c r="B31" s="210"/>
+      <c r="C31" s="196"/>
+      <c r="D31" s="200"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="199"/>
-      <c r="B32" s="198"/>
+      <c r="A32" s="212"/>
+      <c r="B32" s="210"/>
       <c r="C32" s="58" t="s">
         <v>167</v>
       </c>
@@ -6348,8 +6314,8 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="199"/>
-      <c r="B33" s="198"/>
+      <c r="A33" s="212"/>
+      <c r="B33" s="210"/>
       <c r="C33" s="58" t="s">
         <v>168</v>
       </c>
@@ -6358,8 +6324,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="199"/>
-      <c r="B34" s="198"/>
+      <c r="A34" s="212"/>
+      <c r="B34" s="210"/>
       <c r="C34" s="67" t="s">
         <v>170</v>
       </c>
@@ -6368,8 +6334,8 @@
       </c>
     </row>
     <row r="35" spans="1:4" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="199"/>
-      <c r="B35" s="198"/>
+      <c r="A35" s="212"/>
+      <c r="B35" s="210"/>
       <c r="C35" s="58" t="s">
         <v>157</v>
       </c>
@@ -6378,8 +6344,8 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="199"/>
-      <c r="B36" s="198"/>
+      <c r="A36" s="212"/>
+      <c r="B36" s="210"/>
       <c r="C36" s="67" t="s">
         <v>159</v>
       </c>
@@ -6388,26 +6354,26 @@
       </c>
     </row>
     <row r="37" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="199"/>
-      <c r="B37" s="198"/>
-      <c r="C37" s="212" t="s">
+      <c r="A37" s="212"/>
+      <c r="B37" s="210"/>
+      <c r="C37" s="201" t="s">
         <v>161</v>
       </c>
-      <c r="D37" s="214" t="s">
+      <c r="D37" s="203" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="6.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="199"/>
-      <c r="B38" s="198"/>
-      <c r="C38" s="213"/>
-      <c r="D38" s="214"/>
+      <c r="A38" s="212"/>
+      <c r="B38" s="210"/>
+      <c r="C38" s="202"/>
+      <c r="D38" s="203"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="197" t="s">
+      <c r="A39" s="211" t="s">
         <v>86</v>
       </c>
-      <c r="B39" s="198" t="s">
+      <c r="B39" s="210" t="s">
         <v>85</v>
       </c>
       <c r="C39" s="38" t="s">
@@ -6418,8 +6384,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="197"/>
-      <c r="B40" s="198"/>
+      <c r="A40" s="211"/>
+      <c r="B40" s="210"/>
       <c r="C40" s="38"/>
       <c r="D40" s="49" t="s">
         <v>98</v>
@@ -6446,10 +6412,10 @@
       <c r="D42" s="44"/>
     </row>
     <row r="43" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="199" t="s">
+      <c r="A43" s="212" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="198" t="s">
+      <c r="B43" s="210" t="s">
         <v>85</v>
       </c>
       <c r="C43" s="38"/>
@@ -6458,8 +6424,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="199"/>
-      <c r="B44" s="198"/>
+      <c r="A44" s="212"/>
+      <c r="B44" s="210"/>
       <c r="C44" s="38" t="s">
         <v>145</v>
       </c>
@@ -6468,10 +6434,10 @@
       </c>
     </row>
     <row r="45" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="205" t="s">
+      <c r="A45" s="207" t="s">
         <v>80</v>
       </c>
-      <c r="B45" s="198" t="s">
+      <c r="B45" s="210" t="s">
         <v>85</v>
       </c>
       <c r="C45" s="38"/>
@@ -6480,8 +6446,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="206"/>
-      <c r="B46" s="198"/>
+      <c r="A46" s="208"/>
+      <c r="B46" s="210"/>
       <c r="C46" s="38" t="s">
         <v>101</v>
       </c>
@@ -6490,8 +6456,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="206"/>
-      <c r="B47" s="198"/>
+      <c r="A47" s="208"/>
+      <c r="B47" s="210"/>
       <c r="C47" s="38" t="s">
         <v>99</v>
       </c>
@@ -6500,8 +6466,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="207"/>
-      <c r="B48" s="198"/>
+      <c r="A48" s="209"/>
+      <c r="B48" s="210"/>
       <c r="C48" s="38" t="s">
         <v>145</v>
       </c>
@@ -6510,10 +6476,10 @@
       </c>
     </row>
     <row r="49" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A49" s="202" t="s">
+      <c r="A49" s="205" t="s">
         <v>32</v>
       </c>
-      <c r="B49" s="202" t="s">
+      <c r="B49" s="205" t="s">
         <v>85</v>
       </c>
       <c r="C49" s="58"/>
@@ -10617,8 +10583,8 @@
       <c r="XFC49" s="42"/>
     </row>
     <row r="50" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="202"/>
-      <c r="B50" s="202"/>
+      <c r="A50" s="205"/>
+      <c r="B50" s="205"/>
       <c r="C50" s="59" t="s">
         <v>105</v>
       </c>
@@ -14722,8 +14688,8 @@
       <c r="XFC50" s="42"/>
     </row>
     <row r="51" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A51" s="202"/>
-      <c r="B51" s="202"/>
+      <c r="A51" s="205"/>
+      <c r="B51" s="205"/>
       <c r="C51" s="38" t="s">
         <v>107</v>
       </c>
@@ -18827,8 +18793,8 @@
       <c r="XFC51" s="42"/>
     </row>
     <row r="52" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A52" s="202"/>
-      <c r="B52" s="202"/>
+      <c r="A52" s="205"/>
+      <c r="B52" s="205"/>
       <c r="C52" s="58" t="s">
         <v>108</v>
       </c>
@@ -22932,12 +22898,12 @@
       <c r="XFC52" s="42"/>
     </row>
     <row r="53" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A53" s="202"/>
-      <c r="B53" s="202"/>
-      <c r="C53" s="210" t="s">
+      <c r="A53" s="205"/>
+      <c r="B53" s="205"/>
+      <c r="C53" s="199" t="s">
         <v>109</v>
       </c>
-      <c r="D53" s="211" t="s">
+      <c r="D53" s="200" t="s">
         <v>144</v>
       </c>
       <c r="G53" s="42"/>
@@ -27037,10 +27003,10 @@
       <c r="XFC53" s="42"/>
     </row>
     <row r="54" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="202"/>
-      <c r="B54" s="202"/>
-      <c r="C54" s="210"/>
-      <c r="D54" s="211"/>
+      <c r="A54" s="205"/>
+      <c r="B54" s="205"/>
+      <c r="C54" s="199"/>
+      <c r="D54" s="200"/>
       <c r="G54" s="42"/>
       <c r="K54" s="42"/>
       <c r="O54" s="42"/>
@@ -31158,10 +31124,10 @@
       </c>
     </row>
     <row r="57" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A57" s="203" t="s">
+      <c r="A57" s="204" t="s">
         <v>84</v>
       </c>
-      <c r="B57" s="202" t="s">
+      <c r="B57" s="205" t="s">
         <v>85</v>
       </c>
       <c r="C57" s="58" t="s">
@@ -31172,8 +31138,8 @@
       </c>
     </row>
     <row r="58" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="203"/>
-      <c r="B58" s="202"/>
+      <c r="A58" s="204"/>
+      <c r="B58" s="205"/>
       <c r="C58" s="61" t="s">
         <v>113</v>
       </c>
@@ -31182,8 +31148,8 @@
       </c>
     </row>
     <row r="59" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A59" s="203"/>
-      <c r="B59" s="202"/>
+      <c r="A59" s="204"/>
+      <c r="B59" s="205"/>
       <c r="C59" s="58" t="s">
         <v>114</v>
       </c>
@@ -31192,8 +31158,8 @@
       </c>
     </row>
     <row r="60" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" ht="30" x14ac:dyDescent="0.25">
-      <c r="A60" s="203"/>
-      <c r="B60" s="202"/>
+      <c r="A60" s="204"/>
+      <c r="B60" s="205"/>
       <c r="C60" s="58" t="s">
         <v>115</v>
       </c>
@@ -31202,8 +31168,8 @@
       </c>
     </row>
     <row r="61" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A61" s="203"/>
-      <c r="B61" s="202"/>
+      <c r="A61" s="204"/>
+      <c r="B61" s="205"/>
       <c r="C61" s="38" t="s">
         <v>145</v>
       </c>
@@ -31212,8 +31178,8 @@
       </c>
     </row>
     <row r="62" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A62" s="203"/>
-      <c r="B62" s="202"/>
+      <c r="A62" s="204"/>
+      <c r="B62" s="205"/>
       <c r="C62" s="58" t="s">
         <v>117</v>
       </c>
@@ -31222,8 +31188,8 @@
       </c>
     </row>
     <row r="63" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A63" s="203"/>
-      <c r="B63" s="202"/>
+      <c r="A63" s="204"/>
+      <c r="B63" s="205"/>
       <c r="C63" s="58" t="s">
         <v>117</v>
       </c>
@@ -31232,16 +31198,16 @@
       </c>
     </row>
     <row r="64" spans="1:1023 1027:2047 2051:3071 3075:4095 4099:5119 5123:6143 6147:7167 7171:8191 8195:9215 9219:10239 10243:11263 11267:12287 12291:13311 13315:14335 14339:15359 15363:16383" x14ac:dyDescent="0.25">
-      <c r="A64" s="203"/>
-      <c r="B64" s="202"/>
+      <c r="A64" s="204"/>
+      <c r="B64" s="205"/>
       <c r="C64" s="58"/>
       <c r="D64" s="47" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="203"/>
-      <c r="B65" s="202"/>
+      <c r="A65" s="204"/>
+      <c r="B65" s="205"/>
       <c r="C65" s="58" t="s">
         <v>120</v>
       </c>
@@ -31250,16 +31216,16 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="203"/>
-      <c r="B66" s="202"/>
+      <c r="A66" s="204"/>
+      <c r="B66" s="205"/>
       <c r="C66" s="58"/>
       <c r="D66" s="46" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="203"/>
-      <c r="B67" s="202"/>
+      <c r="A67" s="204"/>
+      <c r="B67" s="205"/>
       <c r="C67" s="58" t="s">
         <v>122</v>
       </c>
@@ -31268,8 +31234,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A68" s="203"/>
-      <c r="B68" s="202"/>
+      <c r="A68" s="204"/>
+      <c r="B68" s="205"/>
       <c r="C68" s="58" t="s">
         <v>123</v>
       </c>
@@ -31278,8 +31244,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A69" s="203"/>
-      <c r="B69" s="202"/>
+      <c r="A69" s="204"/>
+      <c r="B69" s="205"/>
       <c r="C69" s="61" t="s">
         <v>125</v>
       </c>
@@ -31288,8 +31254,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A70" s="203"/>
-      <c r="B70" s="202"/>
+      <c r="A70" s="204"/>
+      <c r="B70" s="205"/>
       <c r="C70" s="61" t="s">
         <v>126</v>
       </c>
@@ -31298,8 +31264,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="203"/>
-      <c r="B71" s="202"/>
+      <c r="A71" s="204"/>
+      <c r="B71" s="205"/>
       <c r="C71" s="58" t="s">
         <v>127</v>
       </c>
@@ -31308,8 +31274,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="203"/>
-      <c r="B72" s="202"/>
+      <c r="A72" s="204"/>
+      <c r="B72" s="205"/>
       <c r="C72" s="58" t="s">
         <v>128</v>
       </c>
@@ -31318,16 +31284,16 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="203"/>
-      <c r="B73" s="202"/>
+      <c r="A73" s="204"/>
+      <c r="B73" s="205"/>
       <c r="C73" s="58"/>
       <c r="D73" s="49" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="203"/>
-      <c r="B74" s="202"/>
+      <c r="A74" s="204"/>
+      <c r="B74" s="205"/>
       <c r="C74" s="58" t="s">
         <v>129</v>
       </c>
@@ -31336,18 +31302,18 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="203"/>
-      <c r="B75" s="202"/>
-      <c r="C75" s="209"/>
-      <c r="D75" s="204" t="s">
+      <c r="A75" s="204"/>
+      <c r="B75" s="205"/>
+      <c r="C75" s="198"/>
+      <c r="D75" s="206" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="203"/>
-      <c r="B76" s="202"/>
-      <c r="C76" s="209"/>
-      <c r="D76" s="204"/>
+      <c r="A76" s="204"/>
+      <c r="B76" s="205"/>
+      <c r="C76" s="198"/>
+      <c r="D76" s="206"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="39" t="s">
@@ -31371,8 +31337,8 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}">
-      <selection activeCell="A7" sqref="A7"/>
+    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="A13">
+      <selection activeCell="D20" sqref="D20"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
     </customSheetView>
@@ -31381,29 +31347,13 @@
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
     </customSheetView>
-    <customSheetView guid="{3ECA9ADB-6C26-4D30-9FA0-625C82AEEE29}" topLeftCell="A13">
-      <selection activeCell="D20" sqref="D20"/>
+    <customSheetView guid="{99CEABDF-88F7-4121-AD5F-66FD045725EC}">
+      <selection activeCell="A7" sqref="A7"/>
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
       <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="30">
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="A57:A76"/>
-    <mergeCell ref="B57:B76"/>
-    <mergeCell ref="D75:D76"/>
-    <mergeCell ref="A45:A48"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="A49:A54"/>
-    <mergeCell ref="B49:B54"/>
     <mergeCell ref="A7:A12"/>
     <mergeCell ref="B7:B12"/>
     <mergeCell ref="A43:A44"/>
@@ -31418,6 +31368,22 @@
     <mergeCell ref="B16:B25"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="B39:B40"/>
+    <mergeCell ref="A57:A76"/>
+    <mergeCell ref="B57:B76"/>
+    <mergeCell ref="D75:D76"/>
+    <mergeCell ref="A45:A48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="A49:A54"/>
+    <mergeCell ref="B49:B54"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
@@ -31466,10 +31432,10 @@
       <c r="D3" s="44"/>
     </row>
     <row r="4" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="197" t="s">
+      <c r="A4" s="211" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="198" t="s">
+      <c r="B4" s="210" t="s">
         <v>185</v>
       </c>
       <c r="C4" s="72" t="s">
@@ -31480,133 +31446,133 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="197"/>
-      <c r="B5" s="198"/>
-      <c r="C5" s="224" t="s">
+      <c r="A5" s="211"/>
+      <c r="B5" s="210"/>
+      <c r="C5" s="221" t="s">
         <v>190</v>
       </c>
-      <c r="D5" s="223" t="s">
+      <c r="D5" s="220" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="7.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="197"/>
-      <c r="B6" s="198"/>
-      <c r="C6" s="224"/>
-      <c r="D6" s="223"/>
+      <c r="A6" s="211"/>
+      <c r="B6" s="210"/>
+      <c r="C6" s="221"/>
+      <c r="D6" s="220"/>
     </row>
     <row r="7" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="197"/>
-      <c r="B7" s="198"/>
+      <c r="A7" s="211"/>
+      <c r="B7" s="210"/>
       <c r="C7" s="58"/>
       <c r="D7" s="58"/>
     </row>
     <row r="8" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="197"/>
-      <c r="B8" s="198"/>
+      <c r="A8" s="211"/>
+      <c r="B8" s="210"/>
       <c r="C8" s="58"/>
       <c r="D8" s="58"/>
     </row>
     <row r="9" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="197"/>
-      <c r="B9" s="198"/>
+      <c r="A9" s="211"/>
+      <c r="B9" s="210"/>
       <c r="C9" s="71"/>
       <c r="D9" s="49"/>
     </row>
     <row r="10" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="200" t="s">
+      <c r="A10" s="213" t="s">
         <v>146</v>
       </c>
-      <c r="B10" s="198" t="s">
+      <c r="B10" s="210" t="s">
         <v>185</v>
       </c>
-      <c r="C10" s="222"/>
-      <c r="D10" s="223" t="s">
+      <c r="C10" s="223"/>
+      <c r="D10" s="220" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="200"/>
-      <c r="B11" s="198"/>
-      <c r="C11" s="222"/>
-      <c r="D11" s="223"/>
+      <c r="A11" s="213"/>
+      <c r="B11" s="210"/>
+      <c r="C11" s="223"/>
+      <c r="D11" s="220"/>
     </row>
     <row r="12" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="200"/>
-      <c r="B12" s="198"/>
-      <c r="C12" s="222"/>
-      <c r="D12" s="223"/>
+      <c r="A12" s="213"/>
+      <c r="B12" s="210"/>
+      <c r="C12" s="223"/>
+      <c r="D12" s="220"/>
     </row>
     <row r="13" spans="1:4" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="201" t="s">
+      <c r="A13" s="196" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="202" t="s">
+      <c r="B13" s="205" t="s">
         <v>185</v>
       </c>
-      <c r="C13" s="225"/>
-      <c r="D13" s="223" t="s">
+      <c r="C13" s="222"/>
+      <c r="D13" s="220" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="201"/>
-      <c r="B14" s="202"/>
-      <c r="C14" s="225"/>
-      <c r="D14" s="223"/>
+      <c r="A14" s="196"/>
+      <c r="B14" s="205"/>
+      <c r="C14" s="222"/>
+      <c r="D14" s="220"/>
     </row>
     <row r="15" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="201"/>
-      <c r="B15" s="202"/>
-      <c r="C15" s="225"/>
+      <c r="A15" s="196"/>
+      <c r="B15" s="205"/>
+      <c r="C15" s="222"/>
       <c r="D15" s="49"/>
     </row>
     <row r="16" spans="1:4" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="201"/>
-      <c r="B16" s="202"/>
-      <c r="C16" s="225"/>
+      <c r="A16" s="196"/>
+      <c r="B16" s="205"/>
+      <c r="C16" s="222"/>
       <c r="D16" s="49"/>
     </row>
     <row r="17" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="201"/>
-      <c r="B17" s="202"/>
-      <c r="C17" s="225"/>
+      <c r="A17" s="196"/>
+      <c r="B17" s="205"/>
+      <c r="C17" s="222"/>
       <c r="D17" s="49"/>
     </row>
     <row r="18" spans="1:4" ht="41.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="201"/>
-      <c r="B18" s="202"/>
-      <c r="C18" s="225"/>
+      <c r="A18" s="196"/>
+      <c r="B18" s="205"/>
+      <c r="C18" s="222"/>
       <c r="D18" s="49"/>
     </row>
     <row r="19" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="201"/>
-      <c r="B19" s="202"/>
-      <c r="C19" s="225"/>
+      <c r="A19" s="196"/>
+      <c r="B19" s="205"/>
+      <c r="C19" s="222"/>
       <c r="D19" s="49"/>
     </row>
     <row r="20" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="201"/>
-      <c r="B20" s="202"/>
-      <c r="C20" s="225"/>
+      <c r="A20" s="196"/>
+      <c r="B20" s="205"/>
+      <c r="C20" s="222"/>
       <c r="D20" s="49"/>
     </row>
     <row r="21" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="201"/>
-      <c r="B21" s="202"/>
-      <c r="C21" s="225"/>
+      <c r="A21" s="196"/>
+      <c r="B21" s="205"/>
+      <c r="C21" s="222"/>
       <c r="D21" s="49"/>
     </row>
     <row r="22" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="201"/>
-      <c r="B22" s="202"/>
-      <c r="C22" s="225"/>
+      <c r="A22" s="196"/>
+      <c r="B22" s="205"/>
+      <c r="C22" s="222"/>
       <c r="D22" s="49"/>
     </row>
     <row r="23" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="201"/>
-      <c r="B23" s="202"/>
-      <c r="C23" s="225"/>
+      <c r="A23" s="196"/>
+      <c r="B23" s="205"/>
+      <c r="C23" s="222"/>
       <c r="D23" s="58" t="s">
         <v>221</v>
       </c>
@@ -31704,10 +31670,10 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="226" t="s">
+      <c r="A32" s="214" t="s">
         <v>222</v>
       </c>
-      <c r="B32" s="229" t="s">
+      <c r="B32" s="217" t="s">
         <v>185</v>
       </c>
       <c r="C32" s="91" t="s">
@@ -31718,26 +31684,26 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="227"/>
-      <c r="B33" s="230"/>
+      <c r="A33" s="215"/>
+      <c r="B33" s="218"/>
       <c r="C33" s="78"/>
       <c r="D33" s="75"/>
     </row>
     <row r="34" spans="1:4" ht="9.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="227"/>
-      <c r="B34" s="230"/>
+      <c r="A34" s="215"/>
+      <c r="B34" s="218"/>
       <c r="C34" s="78"/>
       <c r="D34" s="75"/>
     </row>
     <row r="35" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="227"/>
-      <c r="B35" s="230"/>
+      <c r="A35" s="215"/>
+      <c r="B35" s="218"/>
       <c r="C35" s="78"/>
       <c r="D35" s="75"/>
     </row>
     <row r="36" spans="1:4" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="228"/>
-      <c r="B36" s="231"/>
+      <c r="A36" s="216"/>
+      <c r="B36" s="219"/>
       <c r="C36" s="78" t="s">
         <v>223</v>
       </c>
@@ -31766,10 +31732,10 @@
       <c r="D38" s="44"/>
     </row>
     <row r="39" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="199" t="s">
+      <c r="A39" s="212" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="198" t="s">
+      <c r="B39" s="210" t="s">
         <v>185</v>
       </c>
       <c r="C39" s="76" t="s">
@@ -31780,8 +31746,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="199"/>
-      <c r="B40" s="198"/>
+      <c r="A40" s="212"/>
+      <c r="B40" s="210"/>
       <c r="C40" s="69" t="s">
         <v>190</v>
       </c>
@@ -31790,84 +31756,84 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="197" t="s">
+      <c r="A41" s="211" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="198" t="s">
+      <c r="B41" s="210" t="s">
         <v>185</v>
       </c>
-      <c r="C41" s="222" t="s">
+      <c r="C41" s="223" t="s">
         <v>194</v>
       </c>
-      <c r="D41" s="201" t="s">
+      <c r="D41" s="196" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="197"/>
-      <c r="B42" s="198"/>
-      <c r="C42" s="222"/>
-      <c r="D42" s="201"/>
+      <c r="A42" s="211"/>
+      <c r="B42" s="210"/>
+      <c r="C42" s="223"/>
+      <c r="D42" s="196"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="197"/>
-      <c r="B43" s="198"/>
-      <c r="C43" s="222" t="s">
+      <c r="A43" s="211"/>
+      <c r="B43" s="210"/>
+      <c r="C43" s="223" t="s">
         <v>190</v>
       </c>
-      <c r="D43" s="204" t="s">
+      <c r="D43" s="206" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="197"/>
-      <c r="B44" s="198"/>
-      <c r="C44" s="222"/>
-      <c r="D44" s="204"/>
+      <c r="A44" s="211"/>
+      <c r="B44" s="210"/>
+      <c r="C44" s="223"/>
+      <c r="D44" s="206"/>
     </row>
     <row r="45" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="203" t="s">
+      <c r="A45" s="204" t="s">
         <v>32</v>
       </c>
-      <c r="B45" s="202" t="s">
+      <c r="B45" s="205" t="s">
         <v>185</v>
       </c>
-      <c r="C45" s="218"/>
+      <c r="C45" s="227"/>
       <c r="D45" s="90" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="203"/>
-      <c r="B46" s="202"/>
-      <c r="C46" s="219"/>
-      <c r="D46" s="215" t="s">
+      <c r="A46" s="204"/>
+      <c r="B46" s="205"/>
+      <c r="C46" s="228"/>
+      <c r="D46" s="224" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="203"/>
-      <c r="B47" s="202"/>
-      <c r="C47" s="219"/>
-      <c r="D47" s="216"/>
+      <c r="A47" s="204"/>
+      <c r="B47" s="205"/>
+      <c r="C47" s="228"/>
+      <c r="D47" s="225"/>
     </row>
     <row r="48" spans="1:4" ht="13.9" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="203"/>
-      <c r="B48" s="202"/>
-      <c r="C48" s="220"/>
-      <c r="D48" s="216"/>
+      <c r="A48" s="204"/>
+      <c r="B48" s="205"/>
+      <c r="C48" s="229"/>
+      <c r="D48" s="225"/>
     </row>
     <row r="49" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="203"/>
-      <c r="B49" s="202"/>
-      <c r="C49" s="210"/>
-      <c r="D49" s="216"/>
+      <c r="A49" s="204"/>
+      <c r="B49" s="205"/>
+      <c r="C49" s="199"/>
+      <c r="D49" s="225"/>
     </row>
     <row r="50" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="203"/>
-      <c r="B50" s="202"/>
-      <c r="C50" s="210"/>
-      <c r="D50" s="217"/>
+      <c r="A50" s="204"/>
+      <c r="B50" s="205"/>
+      <c r="C50" s="199"/>
+      <c r="D50" s="226"/>
     </row>
     <row r="51" spans="1:4" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="39" t="s">
@@ -31890,10 +31856,10 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="202" t="s">
+      <c r="A53" s="205" t="s">
         <v>84</v>
       </c>
-      <c r="B53" s="202" t="s">
+      <c r="B53" s="205" t="s">
         <v>185</v>
       </c>
       <c r="C53" s="78" t="s">
@@ -31904,8 +31870,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="202"/>
-      <c r="B54" s="202"/>
+      <c r="A54" s="205"/>
+      <c r="B54" s="205"/>
       <c r="C54" s="78" t="s">
         <v>190</v>
       </c>
@@ -31914,8 +31880,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="202"/>
-      <c r="B55" s="202"/>
+      <c r="A55" s="205"/>
+      <c r="B55" s="205"/>
       <c r="C55" s="78" t="s">
         <v>205</v>
       </c>
@@ -31924,9 +31890,9 @@
       </c>
     </row>
     <row r="56" spans="1:4" ht="34.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="202"/>
-      <c r="B56" s="202"/>
-      <c r="C56" s="221" t="s">
+      <c r="A56" s="205"/>
+      <c r="B56" s="205"/>
+      <c r="C56" s="230" t="s">
         <v>208</v>
       </c>
       <c r="D56" s="79" t="s">
@@ -31934,16 +31900,16 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="202"/>
-      <c r="B57" s="202"/>
-      <c r="C57" s="221"/>
+      <c r="A57" s="205"/>
+      <c r="B57" s="205"/>
+      <c r="C57" s="230"/>
       <c r="D57" s="47" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="202"/>
-      <c r="B58" s="202"/>
+      <c r="A58" s="205"/>
+      <c r="B58" s="205"/>
       <c r="C58" s="78" t="s">
         <v>209</v>
       </c>
@@ -31952,8 +31918,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="202"/>
-      <c r="B59" s="202"/>
+      <c r="A59" s="205"/>
+      <c r="B59" s="205"/>
       <c r="C59" s="78" t="s">
         <v>210</v>
       </c>
@@ -31962,9 +31928,9 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="202"/>
-      <c r="B60" s="202"/>
-      <c r="C60" s="221" t="s">
+      <c r="A60" s="205"/>
+      <c r="B60" s="205"/>
+      <c r="C60" s="230" t="s">
         <v>207</v>
       </c>
       <c r="D60" s="46" t="s">
@@ -31972,25 +31938,25 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="202"/>
-      <c r="B61" s="202"/>
-      <c r="C61" s="221"/>
+      <c r="A61" s="205"/>
+      <c r="B61" s="205"/>
+      <c r="C61" s="230"/>
       <c r="D61" s="46" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="202"/>
-      <c r="B62" s="202"/>
-      <c r="C62" s="221"/>
+      <c r="A62" s="205"/>
+      <c r="B62" s="205"/>
+      <c r="C62" s="230"/>
       <c r="D62" s="79" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="202"/>
-      <c r="B63" s="202"/>
-      <c r="C63" s="222" t="s">
+      <c r="A63" s="205"/>
+      <c r="B63" s="205"/>
+      <c r="C63" s="223" t="s">
         <v>206</v>
       </c>
       <c r="D63" s="45" t="s">
@@ -31998,30 +31964,30 @@
       </c>
     </row>
     <row r="64" spans="1:4" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="202"/>
-      <c r="B64" s="202"/>
-      <c r="C64" s="222"/>
-      <c r="D64" s="204" t="s">
+      <c r="A64" s="205"/>
+      <c r="B64" s="205"/>
+      <c r="C64" s="223"/>
+      <c r="D64" s="206" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="12.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="202"/>
-      <c r="B65" s="202"/>
-      <c r="C65" s="222"/>
-      <c r="D65" s="204"/>
+      <c r="A65" s="205"/>
+      <c r="B65" s="205"/>
+      <c r="C65" s="223"/>
+      <c r="D65" s="206"/>
     </row>
     <row r="66" spans="1:4" ht="13.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="202"/>
-      <c r="B66" s="202"/>
-      <c r="C66" s="222"/>
-      <c r="D66" s="204"/>
+      <c r="A66" s="205"/>
+      <c r="B66" s="205"/>
+      <c r="C66" s="223"/>
+      <c r="D66" s="206"/>
     </row>
     <row r="67" spans="1:4" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="202"/>
-      <c r="B67" s="202"/>
-      <c r="C67" s="222"/>
-      <c r="D67" s="204"/>
+      <c r="A67" s="205"/>
+      <c r="B67" s="205"/>
+      <c r="C67" s="223"/>
+      <c r="D67" s="206"/>
     </row>
     <row r="68" spans="1:4" ht="11.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="39"/>
@@ -32077,23 +32043,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A32:A36"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="A4:A9"/>
-    <mergeCell ref="B4:B9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="A13:A23"/>
-    <mergeCell ref="B13:B23"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="C13:C23"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="C43:C44"/>
     <mergeCell ref="D64:D67"/>
     <mergeCell ref="D41:D42"/>
     <mergeCell ref="D46:D50"/>
@@ -32110,6 +32059,23 @@
     <mergeCell ref="B45:B50"/>
     <mergeCell ref="C49:C50"/>
     <mergeCell ref="C63:C67"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="C13:C23"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="A32:A36"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="A4:A9"/>
+    <mergeCell ref="B4:B9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A13:A23"/>
+    <mergeCell ref="B13:B23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -32118,7 +32084,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D298"/>
+  <dimension ref="A1:D294"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="62.42578125" customWidth="1"/>
@@ -32150,10 +32116,10 @@
       <c r="D2" s="104"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="232" t="s">
+      <c r="A3" s="255" t="s">
         <v>434</v>
       </c>
-      <c r="B3" s="232" t="s">
+      <c r="B3" s="255" t="s">
         <v>435</v>
       </c>
       <c r="C3" s="101" t="s">
@@ -32164,8 +32130,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="233"/>
-      <c r="B4" s="233"/>
+      <c r="A4" s="256"/>
+      <c r="B4" s="256"/>
       <c r="C4" s="100" t="s">
         <v>438</v>
       </c>
@@ -32174,8 +32140,8 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="234"/>
-      <c r="B5" s="234"/>
+      <c r="A5" s="257"/>
+      <c r="B5" s="257"/>
       <c r="C5" s="100" t="s">
         <v>438</v>
       </c>
@@ -32198,10 +32164,10 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="232" t="s">
+      <c r="A7" s="255" t="s">
         <v>485</v>
       </c>
-      <c r="B7" s="232" t="s">
+      <c r="B7" s="255" t="s">
         <v>435</v>
       </c>
       <c r="C7" s="141" t="s">
@@ -32212,8 +32178,8 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="233"/>
-      <c r="B8" s="233"/>
+      <c r="A8" s="256"/>
+      <c r="B8" s="256"/>
       <c r="C8" s="141" t="s">
         <v>486</v>
       </c>
@@ -32222,8 +32188,8 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="234"/>
-      <c r="B9" s="234"/>
+      <c r="A9" s="257"/>
+      <c r="B9" s="257"/>
       <c r="C9" s="141" t="s">
         <v>489</v>
       </c>
@@ -32240,7 +32206,7 @@
       <c r="D10" s="127"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="240" t="s">
+      <c r="A11" s="243" t="s">
         <v>248</v>
       </c>
       <c r="B11" s="235" t="s">
@@ -32254,8 +32220,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="241"/>
-      <c r="B12" s="237"/>
+      <c r="A12" s="245"/>
+      <c r="B12" s="236"/>
       <c r="C12" s="128" t="s">
         <v>451</v>
       </c>
@@ -32278,7 +32244,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="236"/>
+      <c r="A14" s="237"/>
       <c r="B14" s="151"/>
       <c r="C14" s="106" t="s">
         <v>300</v>
@@ -32288,7 +32254,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="236"/>
+      <c r="A15" s="237"/>
       <c r="B15" s="151"/>
       <c r="C15" s="128" t="s">
         <v>281</v>
@@ -32298,7 +32264,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="236"/>
+      <c r="A16" s="237"/>
       <c r="B16" s="151"/>
       <c r="C16" s="128" t="s">
         <v>21</v>
@@ -32308,7 +32274,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="236"/>
+      <c r="A17" s="237"/>
       <c r="B17" s="150"/>
       <c r="C17" s="128" t="s">
         <v>449</v>
@@ -32318,7 +32284,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="237"/>
+      <c r="A18" s="236"/>
       <c r="B18" s="151"/>
       <c r="C18" s="128" t="s">
         <v>436</v>
@@ -32342,7 +32308,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="240" t="s">
+      <c r="A20" s="243" t="s">
         <v>454</v>
       </c>
       <c r="B20" s="235" t="s">
@@ -32356,8 +32322,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="241"/>
-      <c r="B21" s="237"/>
+      <c r="A21" s="245"/>
+      <c r="B21" s="236"/>
       <c r="C21" s="128"/>
       <c r="D21" s="106" t="s">
         <v>479</v>
@@ -32372,10 +32338,10 @@
       <c r="D22" s="104"/>
     </row>
     <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="242" t="s">
+      <c r="A23" s="260" t="s">
         <v>337</v>
       </c>
-      <c r="B23" s="243" t="s">
+      <c r="B23" s="261" t="s">
         <v>432</v>
       </c>
       <c r="C23" s="100" t="s">
@@ -32386,8 +32352,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="242"/>
-      <c r="B24" s="243"/>
+      <c r="A24" s="260"/>
+      <c r="B24" s="261"/>
       <c r="C24" s="100" t="s">
         <v>342</v>
       </c>
@@ -32396,8 +32362,8 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="242"/>
-      <c r="B25" s="243"/>
+      <c r="A25" s="260"/>
+      <c r="B25" s="261"/>
       <c r="C25" s="100" t="s">
         <v>338</v>
       </c>
@@ -32414,7 +32380,7 @@
       <c r="D26" s="104"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="240" t="s">
+      <c r="A27" s="243" t="s">
         <v>3</v>
       </c>
       <c r="B27" s="235" t="s">
@@ -32426,8 +32392,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="246"/>
-      <c r="B28" s="236"/>
+      <c r="A28" s="244"/>
+      <c r="B28" s="237"/>
       <c r="C28" s="70" t="s">
         <v>234</v>
       </c>
@@ -32436,8 +32402,8 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="246"/>
-      <c r="B29" s="236"/>
+      <c r="A29" s="244"/>
+      <c r="B29" s="237"/>
       <c r="C29" s="140" t="s">
         <v>445</v>
       </c>
@@ -32446,8 +32412,8 @@
       </c>
     </row>
     <row r="30" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="246"/>
-      <c r="B30" s="236"/>
+      <c r="A30" s="244"/>
+      <c r="B30" s="237"/>
       <c r="C30" s="139" t="s">
         <v>480</v>
       </c>
@@ -32456,8 +32422,8 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="246"/>
-      <c r="B31" s="236"/>
+      <c r="A31" s="244"/>
+      <c r="B31" s="237"/>
       <c r="C31" s="147" t="s">
         <v>491</v>
       </c>
@@ -32466,8 +32432,8 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="246"/>
-      <c r="B32" s="236"/>
+      <c r="A32" s="244"/>
+      <c r="B32" s="237"/>
       <c r="C32" s="147" t="s">
         <v>480</v>
       </c>
@@ -32476,7 +32442,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="240" t="s">
+      <c r="A33" s="243" t="s">
         <v>74</v>
       </c>
       <c r="B33" s="235" t="s">
@@ -32490,8 +32456,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="246"/>
-      <c r="B34" s="236"/>
+      <c r="A34" s="244"/>
+      <c r="B34" s="237"/>
       <c r="C34" s="131" t="s">
         <v>467</v>
       </c>
@@ -32500,8 +32466,8 @@
       </c>
     </row>
     <row r="35" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="241"/>
-      <c r="B35" s="237"/>
+      <c r="A35" s="245"/>
+      <c r="B35" s="236"/>
       <c r="C35" s="136" t="s">
         <v>457</v>
       </c>
@@ -32550,10 +32516,10 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="245" t="s">
+      <c r="A39" s="251" t="s">
         <v>270</v>
       </c>
-      <c r="B39" s="244" t="s">
+      <c r="B39" s="252" t="s">
         <v>432</v>
       </c>
       <c r="C39" s="106"/>
@@ -32562,8 +32528,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="245"/>
-      <c r="B40" s="244"/>
+      <c r="A40" s="251"/>
+      <c r="B40" s="252"/>
       <c r="C40" s="106" t="s">
         <v>494</v>
       </c>
@@ -32572,16 +32538,16 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="245"/>
-      <c r="B41" s="244"/>
+      <c r="A41" s="251"/>
+      <c r="B41" s="252"/>
       <c r="C41" s="106"/>
       <c r="D41" s="106" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="245"/>
-      <c r="B42" s="244"/>
+      <c r="A42" s="251"/>
+      <c r="B42" s="252"/>
       <c r="C42" s="110" t="s">
         <v>320</v>
       </c>
@@ -32590,8 +32556,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="245"/>
-      <c r="B43" s="244"/>
+      <c r="A43" s="251"/>
+      <c r="B43" s="252"/>
       <c r="C43" s="111" t="s">
         <v>399</v>
       </c>
@@ -32612,7 +32578,7 @@
       <c r="D44" s="106"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="238" t="s">
+      <c r="A45" s="258" t="s">
         <v>165</v>
       </c>
       <c r="B45" s="235" t="s">
@@ -32624,8 +32590,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="239"/>
-      <c r="B46" s="236"/>
+      <c r="A46" s="259"/>
+      <c r="B46" s="237"/>
       <c r="C46" s="111" t="s">
         <v>356</v>
       </c>
@@ -32634,8 +32600,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="239"/>
-      <c r="B47" s="236"/>
+      <c r="A47" s="259"/>
+      <c r="B47" s="237"/>
       <c r="C47" s="111" t="s">
         <v>354</v>
       </c>
@@ -32644,8 +32610,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="239"/>
-      <c r="B48" s="236"/>
+      <c r="A48" s="259"/>
+      <c r="B48" s="237"/>
       <c r="C48" s="114" t="s">
         <v>362</v>
       </c>
@@ -32654,8 +32620,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="239"/>
-      <c r="B49" s="236"/>
+      <c r="A49" s="259"/>
+      <c r="B49" s="237"/>
       <c r="C49" s="111" t="s">
         <v>354</v>
       </c>
@@ -32664,8 +32630,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="239"/>
-      <c r="B50" s="236"/>
+      <c r="A50" s="259"/>
+      <c r="B50" s="237"/>
       <c r="C50" s="111" t="s">
         <v>366</v>
       </c>
@@ -32674,8 +32640,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="239"/>
-      <c r="B51" s="236"/>
+      <c r="A51" s="259"/>
+      <c r="B51" s="237"/>
       <c r="C51" s="111" t="s">
         <v>354</v>
       </c>
@@ -32684,8 +32650,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="239"/>
-      <c r="B52" s="236"/>
+      <c r="A52" s="259"/>
+      <c r="B52" s="237"/>
       <c r="C52" s="130" t="s">
         <v>461</v>
       </c>
@@ -32694,8 +32660,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="239"/>
-      <c r="B53" s="236"/>
+      <c r="A53" s="259"/>
+      <c r="B53" s="237"/>
       <c r="C53" s="130" t="s">
         <v>456</v>
       </c>
@@ -32704,8 +32670,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="239"/>
-      <c r="B54" s="236"/>
+      <c r="A54" s="259"/>
+      <c r="B54" s="237"/>
       <c r="C54" s="130" t="s">
         <v>354</v>
       </c>
@@ -32714,8 +32680,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="239"/>
-      <c r="B55" s="236"/>
+      <c r="A55" s="259"/>
+      <c r="B55" s="237"/>
       <c r="C55" s="130" t="s">
         <v>456</v>
       </c>
@@ -32724,8 +32690,8 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="239"/>
-      <c r="B56" s="236"/>
+      <c r="A56" s="259"/>
+      <c r="B56" s="237"/>
       <c r="C56" s="145" t="s">
         <v>354</v>
       </c>
@@ -32734,8 +32700,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="239"/>
-      <c r="B57" s="236"/>
+      <c r="A57" s="259"/>
+      <c r="B57" s="237"/>
       <c r="C57" s="145" t="s">
         <v>480</v>
       </c>
@@ -32744,8 +32710,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="239"/>
-      <c r="B58" s="236"/>
+      <c r="A58" s="259"/>
+      <c r="B58" s="237"/>
       <c r="C58" s="147" t="s">
         <v>491</v>
       </c>
@@ -32754,8 +32720,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="239"/>
-      <c r="B59" s="236"/>
+      <c r="A59" s="259"/>
+      <c r="B59" s="237"/>
       <c r="C59" s="147" t="s">
         <v>480</v>
       </c>
@@ -32790,7 +32756,7 @@
       <c r="D61" s="112"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="247" t="s">
+      <c r="A62" s="233" t="s">
         <v>364</v>
       </c>
       <c r="B62" s="235" t="s">
@@ -32802,8 +32768,8 @@
       <c r="D62" s="112"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="260"/>
-      <c r="B63" s="237"/>
+      <c r="A63" s="234"/>
+      <c r="B63" s="236"/>
       <c r="C63" s="111" t="s">
         <v>399</v>
       </c>
@@ -32820,7 +32786,7 @@
       <c r="D64" s="103"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="247" t="s">
+      <c r="A65" s="233" t="s">
         <v>236</v>
       </c>
       <c r="B65" s="235" t="s">
@@ -32832,24 +32798,24 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="248"/>
-      <c r="B66" s="236"/>
+      <c r="A66" s="246"/>
+      <c r="B66" s="237"/>
       <c r="C66" s="106"/>
       <c r="D66" s="106" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="248"/>
-      <c r="B67" s="236"/>
+      <c r="A67" s="246"/>
+      <c r="B67" s="237"/>
       <c r="C67" s="106"/>
       <c r="D67" s="106" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="248"/>
-      <c r="B68" s="236"/>
+      <c r="A68" s="246"/>
+      <c r="B68" s="237"/>
       <c r="C68" s="106" t="s">
         <v>295</v>
       </c>
@@ -32858,8 +32824,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="248"/>
-      <c r="B69" s="236"/>
+      <c r="A69" s="246"/>
+      <c r="B69" s="237"/>
       <c r="C69" s="106" t="s">
         <v>323</v>
       </c>
@@ -32868,8 +32834,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="248"/>
-      <c r="B70" s="236"/>
+      <c r="A70" s="246"/>
+      <c r="B70" s="237"/>
       <c r="C70" s="106" t="s">
         <v>368</v>
       </c>
@@ -32878,8 +32844,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="248"/>
-      <c r="B71" s="236"/>
+      <c r="A71" s="246"/>
+      <c r="B71" s="237"/>
       <c r="C71" s="61" t="s">
         <v>472</v>
       </c>
@@ -32888,8 +32854,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="248"/>
-      <c r="B72" s="236"/>
+      <c r="A72" s="246"/>
+      <c r="B72" s="237"/>
       <c r="C72" s="58" t="s">
         <v>37</v>
       </c>
@@ -32898,8 +32864,8 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="248"/>
-      <c r="B73" s="236"/>
+      <c r="A73" s="246"/>
+      <c r="B73" s="237"/>
       <c r="C73" s="137" t="s">
         <v>354</v>
       </c>
@@ -32908,8 +32874,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="248"/>
-      <c r="B74" s="236"/>
+      <c r="A74" s="246"/>
+      <c r="B74" s="237"/>
       <c r="C74" s="137" t="s">
         <v>456</v>
       </c>
@@ -32918,8 +32884,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="248"/>
-      <c r="B75" s="236"/>
+      <c r="A75" s="246"/>
+      <c r="B75" s="237"/>
       <c r="C75" s="137" t="s">
         <v>480</v>
       </c>
@@ -32928,8 +32894,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="248"/>
-      <c r="B76" s="236"/>
+      <c r="A76" s="246"/>
+      <c r="B76" s="237"/>
       <c r="C76" s="146" t="s">
         <v>491</v>
       </c>
@@ -32938,8 +32904,8 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="248"/>
-      <c r="B77" s="236"/>
+      <c r="A77" s="246"/>
+      <c r="B77" s="237"/>
       <c r="C77" s="146" t="s">
         <v>480</v>
       </c>
@@ -32948,7 +32914,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="250" t="s">
+      <c r="A78" s="247" t="s">
         <v>27</v>
       </c>
       <c r="B78" s="235" t="s">
@@ -32962,16 +32928,16 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="251"/>
-      <c r="B79" s="236"/>
+      <c r="A79" s="248"/>
+      <c r="B79" s="237"/>
       <c r="C79" s="106"/>
       <c r="D79" s="106" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A80" s="251"/>
-      <c r="B80" s="236"/>
+      <c r="A80" s="248"/>
+      <c r="B80" s="237"/>
       <c r="C80" s="116" t="s">
         <v>324</v>
       </c>
@@ -32980,8 +32946,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="251"/>
-      <c r="B81" s="236"/>
+      <c r="A81" s="248"/>
+      <c r="B81" s="237"/>
       <c r="C81" s="116" t="s">
         <v>494</v>
       </c>
@@ -32990,8 +32956,8 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="251"/>
-      <c r="B82" s="236"/>
+      <c r="A82" s="248"/>
+      <c r="B82" s="237"/>
       <c r="C82" s="116" t="s">
         <v>354</v>
       </c>
@@ -33000,8 +32966,8 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="251"/>
-      <c r="B83" s="236"/>
+      <c r="A83" s="248"/>
+      <c r="B83" s="237"/>
       <c r="C83" s="116" t="s">
         <v>362</v>
       </c>
@@ -33010,8 +32976,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="251"/>
-      <c r="B84" s="236"/>
+      <c r="A84" s="248"/>
+      <c r="B84" s="237"/>
       <c r="C84" s="116" t="s">
         <v>366</v>
       </c>
@@ -33020,8 +32986,8 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="251"/>
-      <c r="B85" s="236"/>
+      <c r="A85" s="248"/>
+      <c r="B85" s="237"/>
       <c r="C85" s="116" t="s">
         <v>376</v>
       </c>
@@ -33030,8 +32996,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="251"/>
-      <c r="B86" s="236"/>
+      <c r="A86" s="248"/>
+      <c r="B86" s="237"/>
       <c r="C86" s="108" t="s">
         <v>354</v>
       </c>
@@ -33040,8 +33006,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="251"/>
-      <c r="B87" s="236"/>
+      <c r="A87" s="248"/>
+      <c r="B87" s="237"/>
       <c r="C87" s="137" t="s">
         <v>461</v>
       </c>
@@ -33050,8 +33016,8 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="251"/>
-      <c r="B88" s="236"/>
+      <c r="A88" s="248"/>
+      <c r="B88" s="237"/>
       <c r="C88" s="137" t="s">
         <v>456</v>
       </c>
@@ -33060,8 +33026,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="251"/>
-      <c r="B89" s="236"/>
+      <c r="A89" s="248"/>
+      <c r="B89" s="237"/>
       <c r="C89" s="137" t="s">
         <v>354</v>
       </c>
@@ -33070,8 +33036,8 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="251"/>
-      <c r="B90" s="236"/>
+      <c r="A90" s="248"/>
+      <c r="B90" s="237"/>
       <c r="C90" s="137" t="s">
         <v>456</v>
       </c>
@@ -33080,8 +33046,8 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="251"/>
-      <c r="B91" s="236"/>
+      <c r="A91" s="248"/>
+      <c r="B91" s="237"/>
       <c r="C91" s="137" t="s">
         <v>368</v>
       </c>
@@ -33090,8 +33056,8 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="251"/>
-      <c r="B92" s="236"/>
+      <c r="A92" s="248"/>
+      <c r="B92" s="237"/>
       <c r="C92" s="137" t="s">
         <v>354</v>
       </c>
@@ -33100,8 +33066,8 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="251"/>
-      <c r="B93" s="236"/>
+      <c r="A93" s="248"/>
+      <c r="B93" s="237"/>
       <c r="C93" s="137" t="s">
         <v>480</v>
       </c>
@@ -33110,8 +33076,8 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="251"/>
-      <c r="B94" s="236"/>
+      <c r="A94" s="248"/>
+      <c r="B94" s="237"/>
       <c r="C94" s="146" t="s">
         <v>491</v>
       </c>
@@ -33120,8 +33086,8 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="252"/>
-      <c r="B95" s="237"/>
+      <c r="A95" s="249"/>
+      <c r="B95" s="236"/>
       <c r="C95" s="146" t="s">
         <v>480</v>
       </c>
@@ -33130,7 +33096,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="240" t="s">
+      <c r="A96" s="243" t="s">
         <v>222</v>
       </c>
       <c r="B96" s="235" t="s">
@@ -33144,17 +33110,17 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="246"/>
-      <c r="B97" s="236"/>
+      <c r="A97" s="244"/>
+      <c r="B97" s="237"/>
       <c r="C97" s="254"/>
       <c r="D97" s="112" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="246"/>
-      <c r="B98" s="236"/>
-      <c r="C98" s="249" t="s">
+      <c r="A98" s="244"/>
+      <c r="B98" s="237"/>
+      <c r="C98" s="250" t="s">
         <v>239</v>
       </c>
       <c r="D98" s="106" t="s">
@@ -33162,16 +33128,16 @@
       </c>
     </row>
     <row r="99" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A99" s="246"/>
-      <c r="B99" s="236"/>
-      <c r="C99" s="249"/>
+      <c r="A99" s="244"/>
+      <c r="B99" s="237"/>
+      <c r="C99" s="250"/>
       <c r="D99" s="118" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="246"/>
-      <c r="B100" s="236"/>
+      <c r="A100" s="244"/>
+      <c r="B100" s="237"/>
       <c r="C100" s="111" t="s">
         <v>302</v>
       </c>
@@ -33180,8 +33146,8 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="246"/>
-      <c r="B101" s="236"/>
+      <c r="A101" s="244"/>
+      <c r="B101" s="237"/>
       <c r="C101" s="111">
         <v>2.1</v>
       </c>
@@ -33190,8 +33156,8 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="246"/>
-      <c r="B102" s="236"/>
+      <c r="A102" s="244"/>
+      <c r="B102" s="237"/>
       <c r="C102" s="111" t="s">
         <v>238</v>
       </c>
@@ -33200,8 +33166,8 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="246"/>
-      <c r="B103" s="236"/>
+      <c r="A103" s="244"/>
+      <c r="B103" s="237"/>
       <c r="C103" s="111" t="s">
         <v>238</v>
       </c>
@@ -33210,8 +33176,8 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="246"/>
-      <c r="B104" s="236"/>
+      <c r="A104" s="244"/>
+      <c r="B104" s="237"/>
       <c r="C104" s="111" t="s">
         <v>238</v>
       </c>
@@ -33220,8 +33186,8 @@
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="246"/>
-      <c r="B105" s="236"/>
+      <c r="A105" s="244"/>
+      <c r="B105" s="237"/>
       <c r="C105" s="119" t="s">
         <v>373</v>
       </c>
@@ -33230,8 +33196,8 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="246"/>
-      <c r="B106" s="236"/>
+      <c r="A106" s="244"/>
+      <c r="B106" s="237"/>
       <c r="C106" s="111">
         <v>2.1</v>
       </c>
@@ -33240,8 +33206,8 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="246"/>
-      <c r="B107" s="236"/>
+      <c r="A107" s="244"/>
+      <c r="B107" s="237"/>
       <c r="C107" s="111" t="s">
         <v>238</v>
       </c>
@@ -33250,8 +33216,8 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="246"/>
-      <c r="B108" s="236"/>
+      <c r="A108" s="244"/>
+      <c r="B108" s="237"/>
       <c r="C108" s="111" t="s">
         <v>238</v>
       </c>
@@ -33260,8 +33226,8 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="246"/>
-      <c r="B109" s="236"/>
+      <c r="A109" s="244"/>
+      <c r="B109" s="237"/>
       <c r="C109" s="111">
         <v>2.1</v>
       </c>
@@ -33270,7 +33236,7 @@
       </c>
     </row>
     <row r="110" spans="1:4" ht="30.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="250" t="s">
+      <c r="A110" s="247" t="s">
         <v>291</v>
       </c>
       <c r="B110" s="235" t="s">
@@ -33284,8 +33250,8 @@
       </c>
     </row>
     <row r="111" spans="1:4" ht="30.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="251"/>
-      <c r="B111" s="236"/>
+      <c r="A111" s="248"/>
+      <c r="B111" s="237"/>
       <c r="C111" s="106" t="s">
         <v>494</v>
       </c>
@@ -33294,8 +33260,8 @@
       </c>
     </row>
     <row r="112" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A112" s="251"/>
-      <c r="B112" s="236"/>
+      <c r="A112" s="248"/>
+      <c r="B112" s="237"/>
       <c r="C112" s="118" t="s">
         <v>276</v>
       </c>
@@ -33304,8 +33270,8 @@
       </c>
     </row>
     <row r="113" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="252"/>
-      <c r="B113" s="237"/>
+      <c r="A113" s="249"/>
+      <c r="B113" s="236"/>
       <c r="C113" s="106" t="s">
         <v>345</v>
       </c>
@@ -33314,7 +33280,7 @@
       </c>
     </row>
     <row r="114" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="247" t="s">
+      <c r="A114" s="233" t="s">
         <v>365</v>
       </c>
       <c r="B114" s="235" t="s">
@@ -33326,8 +33292,8 @@
       <c r="D114" s="106"/>
     </row>
     <row r="115" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="248"/>
-      <c r="B115" s="236"/>
+      <c r="A115" s="246"/>
+      <c r="B115" s="237"/>
       <c r="C115" s="111" t="s">
         <v>373</v>
       </c>
@@ -33336,8 +33302,8 @@
       </c>
     </row>
     <row r="116" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="248"/>
-      <c r="B116" s="236"/>
+      <c r="A116" s="246"/>
+      <c r="B116" s="237"/>
       <c r="C116" s="111">
         <v>2.1</v>
       </c>
@@ -33346,8 +33312,8 @@
       </c>
     </row>
     <row r="117" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="248"/>
-      <c r="B117" s="236"/>
+      <c r="A117" s="246"/>
+      <c r="B117" s="237"/>
       <c r="C117" s="111" t="s">
         <v>239</v>
       </c>
@@ -33356,8 +33322,8 @@
       </c>
     </row>
     <row r="118" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="248"/>
-      <c r="B118" s="236"/>
+      <c r="A118" s="246"/>
+      <c r="B118" s="237"/>
       <c r="C118" s="111" t="s">
         <v>238</v>
       </c>
@@ -33386,7 +33352,7 @@
       <c r="D120" s="112"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" s="240" t="s">
+      <c r="A121" s="243" t="s">
         <v>256</v>
       </c>
       <c r="B121" s="235" t="s">
@@ -33398,24 +33364,24 @@
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" s="246"/>
-      <c r="B122" s="236"/>
+      <c r="A122" s="244"/>
+      <c r="B122" s="237"/>
       <c r="C122" s="106"/>
       <c r="D122" s="106" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" s="246"/>
-      <c r="B123" s="236"/>
+      <c r="A123" s="244"/>
+      <c r="B123" s="237"/>
       <c r="C123" s="106"/>
       <c r="D123" s="112" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A124" s="246"/>
-      <c r="B124" s="236"/>
+      <c r="A124" s="244"/>
+      <c r="B124" s="237"/>
       <c r="C124" s="106" t="s">
         <v>419</v>
       </c>
@@ -33424,8 +33390,8 @@
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" s="246"/>
-      <c r="B125" s="236"/>
+      <c r="A125" s="244"/>
+      <c r="B125" s="237"/>
       <c r="C125" s="106" t="s">
         <v>424</v>
       </c>
@@ -33434,8 +33400,8 @@
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" s="246"/>
-      <c r="B126" s="236"/>
+      <c r="A126" s="244"/>
+      <c r="B126" s="237"/>
       <c r="C126" s="58" t="s">
         <v>474</v>
       </c>
@@ -33444,8 +33410,8 @@
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A127" s="246"/>
-      <c r="B127" s="236"/>
+      <c r="A127" s="244"/>
+      <c r="B127" s="237"/>
       <c r="C127" s="58" t="s">
         <v>480</v>
       </c>
@@ -33454,10 +33420,10 @@
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="245" t="s">
+      <c r="A128" s="251" t="s">
         <v>329</v>
       </c>
-      <c r="B128" s="244" t="s">
+      <c r="B128" s="252" t="s">
         <v>432</v>
       </c>
       <c r="C128" s="80" t="s">
@@ -33468,8 +33434,8 @@
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A129" s="245"/>
-      <c r="B129" s="244"/>
+      <c r="A129" s="251"/>
+      <c r="B129" s="252"/>
       <c r="C129" s="106" t="s">
         <v>406</v>
       </c>
@@ -33478,42 +33444,42 @@
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A130" s="245"/>
-      <c r="B130" s="244"/>
+      <c r="A130" s="251"/>
+      <c r="B130" s="252"/>
       <c r="C130" s="121" t="s">
         <v>409</v>
       </c>
-      <c r="D130" s="247" t="s">
+      <c r="D130" s="233" t="s">
         <v>413</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A131" s="245"/>
-      <c r="B131" s="244"/>
+      <c r="A131" s="251"/>
+      <c r="B131" s="252"/>
       <c r="C131" s="121" t="s">
         <v>410</v>
       </c>
-      <c r="D131" s="248"/>
+      <c r="D131" s="246"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A132" s="245"/>
-      <c r="B132" s="244"/>
+      <c r="A132" s="251"/>
+      <c r="B132" s="252"/>
       <c r="C132" s="121" t="s">
         <v>411</v>
       </c>
-      <c r="D132" s="248"/>
+      <c r="D132" s="246"/>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A133" s="245"/>
-      <c r="B133" s="244"/>
+      <c r="A133" s="251"/>
+      <c r="B133" s="252"/>
       <c r="C133" s="121" t="s">
         <v>412</v>
       </c>
-      <c r="D133" s="248"/>
+      <c r="D133" s="246"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A134" s="245"/>
-      <c r="B134" s="244"/>
+      <c r="A134" s="251"/>
+      <c r="B134" s="252"/>
       <c r="C134" s="138" t="s">
         <v>475</v>
       </c>
@@ -33536,7 +33502,7 @@
       </c>
     </row>
     <row r="136" spans="1:4" ht="30.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="255" t="s">
+      <c r="A136" s="238" t="s">
         <v>32</v>
       </c>
       <c r="B136" s="235" t="s">
@@ -33550,8 +33516,8 @@
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A137" s="256"/>
-      <c r="B137" s="236"/>
+      <c r="A137" s="239"/>
+      <c r="B137" s="237"/>
       <c r="C137" s="106" t="s">
         <v>265</v>
       </c>
@@ -33560,8 +33526,8 @@
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A138" s="256"/>
-      <c r="B138" s="236"/>
+      <c r="A138" s="239"/>
+      <c r="B138" s="237"/>
       <c r="C138" s="106" t="s">
         <v>264</v>
       </c>
@@ -33570,8 +33536,8 @@
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A139" s="256"/>
-      <c r="B139" s="236"/>
+      <c r="A139" s="239"/>
+      <c r="B139" s="237"/>
       <c r="C139" s="112" t="s">
         <v>272</v>
       </c>
@@ -33580,8 +33546,8 @@
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A140" s="256"/>
-      <c r="B140" s="236"/>
+      <c r="A140" s="239"/>
+      <c r="B140" s="237"/>
       <c r="C140" s="106" t="s">
         <v>277</v>
       </c>
@@ -33590,8 +33556,8 @@
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A141" s="256"/>
-      <c r="B141" s="236"/>
+      <c r="A141" s="239"/>
+      <c r="B141" s="237"/>
       <c r="C141" s="106" t="s">
         <v>278</v>
       </c>
@@ -33600,8 +33566,8 @@
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A142" s="256"/>
-      <c r="B142" s="236"/>
+      <c r="A142" s="239"/>
+      <c r="B142" s="237"/>
       <c r="C142" s="112" t="s">
         <v>283</v>
       </c>
@@ -33610,8 +33576,8 @@
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A143" s="256"/>
-      <c r="B143" s="236"/>
+      <c r="A143" s="239"/>
+      <c r="B143" s="237"/>
       <c r="C143" s="112" t="s">
         <v>297</v>
       </c>
@@ -33620,8 +33586,8 @@
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A144" s="256"/>
-      <c r="B144" s="236"/>
+      <c r="A144" s="239"/>
+      <c r="B144" s="237"/>
       <c r="C144" s="112" t="s">
         <v>284</v>
       </c>
@@ -33630,8 +33596,8 @@
       </c>
     </row>
     <row r="145" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A145" s="256"/>
-      <c r="B145" s="236"/>
+      <c r="A145" s="239"/>
+      <c r="B145" s="237"/>
       <c r="C145" s="122" t="s">
         <v>243</v>
       </c>
@@ -33640,8 +33606,8 @@
       </c>
     </row>
     <row r="146" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A146" s="256"/>
-      <c r="B146" s="236"/>
+      <c r="A146" s="239"/>
+      <c r="B146" s="237"/>
       <c r="C146" s="116" t="s">
         <v>306</v>
       </c>
@@ -33650,8 +33616,8 @@
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A147" s="256"/>
-      <c r="B147" s="236"/>
+      <c r="A147" s="239"/>
+      <c r="B147" s="237"/>
       <c r="C147" s="106" t="s">
         <v>307</v>
       </c>
@@ -33660,8 +33626,8 @@
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A148" s="256"/>
-      <c r="B148" s="236"/>
+      <c r="A148" s="239"/>
+      <c r="B148" s="237"/>
       <c r="C148" s="112" t="s">
         <v>308</v>
       </c>
@@ -33670,8 +33636,8 @@
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" s="256"/>
-      <c r="B149" s="236"/>
+      <c r="A149" s="239"/>
+      <c r="B149" s="237"/>
       <c r="C149" s="112" t="s">
         <v>310</v>
       </c>
@@ -33680,8 +33646,8 @@
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A150" s="256"/>
-      <c r="B150" s="236"/>
+      <c r="A150" s="239"/>
+      <c r="B150" s="237"/>
       <c r="C150" s="112" t="s">
         <v>263</v>
       </c>
@@ -33690,8 +33656,8 @@
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A151" s="256"/>
-      <c r="B151" s="236"/>
+      <c r="A151" s="239"/>
+      <c r="B151" s="237"/>
       <c r="C151" s="106" t="s">
         <v>313</v>
       </c>
@@ -33700,8 +33666,8 @@
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A152" s="256"/>
-      <c r="B152" s="236"/>
+      <c r="A152" s="239"/>
+      <c r="B152" s="237"/>
       <c r="C152" s="112" t="s">
         <v>278</v>
       </c>
@@ -33710,8 +33676,8 @@
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A153" s="256"/>
-      <c r="B153" s="236"/>
+      <c r="A153" s="239"/>
+      <c r="B153" s="237"/>
       <c r="C153" s="112" t="s">
         <v>314</v>
       </c>
@@ -33720,16 +33686,16 @@
       </c>
     </row>
     <row r="154" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A154" s="256"/>
-      <c r="B154" s="236"/>
+      <c r="A154" s="239"/>
+      <c r="B154" s="237"/>
       <c r="C154" s="106"/>
       <c r="D154" s="97" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A155" s="256"/>
-      <c r="B155" s="236"/>
+      <c r="A155" s="239"/>
+      <c r="B155" s="237"/>
       <c r="C155" s="112" t="s">
         <v>317</v>
       </c>
@@ -33738,8 +33704,8 @@
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A156" s="256"/>
-      <c r="B156" s="236"/>
+      <c r="A156" s="239"/>
+      <c r="B156" s="237"/>
       <c r="C156" s="112" t="s">
         <v>263</v>
       </c>
@@ -33748,8 +33714,8 @@
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A157" s="256"/>
-      <c r="B157" s="236"/>
+      <c r="A157" s="239"/>
+      <c r="B157" s="237"/>
       <c r="C157" s="112" t="s">
         <v>334</v>
       </c>
@@ -33758,8 +33724,8 @@
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A158" s="256"/>
-      <c r="B158" s="236"/>
+      <c r="A158" s="239"/>
+      <c r="B158" s="237"/>
       <c r="C158" s="112" t="s">
         <v>335</v>
       </c>
@@ -33768,8 +33734,8 @@
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A159" s="256"/>
-      <c r="B159" s="236"/>
+      <c r="A159" s="239"/>
+      <c r="B159" s="237"/>
       <c r="C159" s="112" t="s">
         <v>319</v>
       </c>
@@ -33778,8 +33744,8 @@
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A160" s="256"/>
-      <c r="B160" s="236"/>
+      <c r="A160" s="239"/>
+      <c r="B160" s="237"/>
       <c r="C160" s="117" t="s">
         <v>340</v>
       </c>
@@ -33788,8 +33754,8 @@
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A161" s="256"/>
-      <c r="B161" s="236"/>
+      <c r="A161" s="239"/>
+      <c r="B161" s="237"/>
       <c r="C161" s="112" t="s">
         <v>333</v>
       </c>
@@ -33798,8 +33764,8 @@
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A162" s="256"/>
-      <c r="B162" s="236"/>
+      <c r="A162" s="239"/>
+      <c r="B162" s="237"/>
       <c r="C162" s="112" t="s">
         <v>348</v>
       </c>
@@ -33808,8 +33774,8 @@
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A163" s="256"/>
-      <c r="B163" s="236"/>
+      <c r="A163" s="239"/>
+      <c r="B163" s="237"/>
       <c r="C163" s="101" t="s">
         <v>351</v>
       </c>
@@ -33818,8 +33784,8 @@
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A164" s="256"/>
-      <c r="B164" s="236"/>
+      <c r="A164" s="239"/>
+      <c r="B164" s="237"/>
       <c r="C164" s="112" t="s">
         <v>352</v>
       </c>
@@ -33828,8 +33794,8 @@
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A165" s="256"/>
-      <c r="B165" s="236"/>
+      <c r="A165" s="239"/>
+      <c r="B165" s="237"/>
       <c r="C165" s="112" t="s">
         <v>353</v>
       </c>
@@ -33838,8 +33804,8 @@
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A166" s="256"/>
-      <c r="B166" s="236"/>
+      <c r="A166" s="239"/>
+      <c r="B166" s="237"/>
       <c r="C166" s="112" t="s">
         <v>359</v>
       </c>
@@ -33848,8 +33814,8 @@
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A167" s="256"/>
-      <c r="B167" s="236"/>
+      <c r="A167" s="239"/>
+      <c r="B167" s="237"/>
       <c r="C167" s="112" t="s">
         <v>361</v>
       </c>
@@ -33858,8 +33824,8 @@
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A168" s="256"/>
-      <c r="B168" s="236"/>
+      <c r="A168" s="239"/>
+      <c r="B168" s="237"/>
       <c r="C168" s="112" t="s">
         <v>367</v>
       </c>
@@ -33868,8 +33834,8 @@
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A169" s="256"/>
-      <c r="B169" s="236"/>
+      <c r="A169" s="239"/>
+      <c r="B169" s="237"/>
       <c r="C169" s="112" t="s">
         <v>359</v>
       </c>
@@ -33878,8 +33844,8 @@
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A170" s="256"/>
-      <c r="B170" s="236"/>
+      <c r="A170" s="239"/>
+      <c r="B170" s="237"/>
       <c r="C170" s="117" t="s">
         <v>380</v>
       </c>
@@ -33888,8 +33854,8 @@
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A171" s="256"/>
-      <c r="B171" s="236"/>
+      <c r="A171" s="239"/>
+      <c r="B171" s="237"/>
       <c r="C171" s="106" t="s">
         <v>384</v>
       </c>
@@ -33898,8 +33864,8 @@
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A172" s="256"/>
-      <c r="B172" s="236"/>
+      <c r="A172" s="239"/>
+      <c r="B172" s="237"/>
       <c r="C172" s="106" t="s">
         <v>387</v>
       </c>
@@ -33908,8 +33874,8 @@
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A173" s="256"/>
-      <c r="B173" s="236"/>
+      <c r="A173" s="239"/>
+      <c r="B173" s="237"/>
       <c r="C173" s="106" t="s">
         <v>388</v>
       </c>
@@ -33918,8 +33884,8 @@
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A174" s="256"/>
-      <c r="B174" s="236"/>
+      <c r="A174" s="239"/>
+      <c r="B174" s="237"/>
       <c r="C174" s="106" t="s">
         <v>389</v>
       </c>
@@ -33928,8 +33894,8 @@
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A175" s="256"/>
-      <c r="B175" s="236"/>
+      <c r="A175" s="239"/>
+      <c r="B175" s="237"/>
       <c r="C175" s="106" t="s">
         <v>390</v>
       </c>
@@ -33938,8 +33904,8 @@
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A176" s="256"/>
-      <c r="B176" s="236"/>
+      <c r="A176" s="239"/>
+      <c r="B176" s="237"/>
       <c r="C176" s="106" t="s">
         <v>391</v>
       </c>
@@ -33948,8 +33914,8 @@
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A177" s="256"/>
-      <c r="B177" s="236"/>
+      <c r="A177" s="239"/>
+      <c r="B177" s="237"/>
       <c r="C177" s="106" t="s">
         <v>394</v>
       </c>
@@ -33958,8 +33924,8 @@
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A178" s="256"/>
-      <c r="B178" s="236"/>
+      <c r="A178" s="239"/>
+      <c r="B178" s="237"/>
       <c r="C178" s="106" t="s">
         <v>404</v>
       </c>
@@ -33968,8 +33934,8 @@
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A179" s="256"/>
-      <c r="B179" s="236"/>
+      <c r="A179" s="239"/>
+      <c r="B179" s="237"/>
       <c r="C179" s="106" t="s">
         <v>405</v>
       </c>
@@ -33978,8 +33944,8 @@
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A180" s="256"/>
-      <c r="B180" s="236"/>
+      <c r="A180" s="239"/>
+      <c r="B180" s="237"/>
       <c r="C180" s="106" t="s">
         <v>422</v>
       </c>
@@ -33988,8 +33954,8 @@
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A181" s="256"/>
-      <c r="B181" s="236"/>
+      <c r="A181" s="239"/>
+      <c r="B181" s="237"/>
       <c r="C181" s="106" t="s">
         <v>423</v>
       </c>
@@ -33998,8 +33964,8 @@
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A182" s="256"/>
-      <c r="B182" s="236"/>
+      <c r="A182" s="239"/>
+      <c r="B182" s="237"/>
       <c r="C182" s="106" t="s">
         <v>426</v>
       </c>
@@ -34008,8 +33974,8 @@
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A183" s="256"/>
-      <c r="B183" s="236"/>
+      <c r="A183" s="239"/>
+      <c r="B183" s="237"/>
       <c r="C183" s="58" t="s">
         <v>477</v>
       </c>
@@ -34018,8 +33984,8 @@
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A184" s="256"/>
-      <c r="B184" s="236"/>
+      <c r="A184" s="239"/>
+      <c r="B184" s="237"/>
       <c r="C184" s="106" t="s">
         <v>422</v>
       </c>
@@ -34028,8 +33994,8 @@
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A185" s="256"/>
-      <c r="B185" s="236"/>
+      <c r="A185" s="239"/>
+      <c r="B185" s="237"/>
       <c r="C185" s="106" t="s">
         <v>476</v>
       </c>
@@ -34038,8 +34004,8 @@
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A186" s="257"/>
-      <c r="B186" s="237"/>
+      <c r="A186" s="240"/>
+      <c r="B186" s="236"/>
       <c r="C186" s="112" t="s">
         <v>333</v>
       </c>
@@ -34048,7 +34014,7 @@
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A187" s="255" t="s">
+      <c r="A187" s="238" t="s">
         <v>416</v>
       </c>
       <c r="B187" s="235" t="s">
@@ -34062,8 +34028,8 @@
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A188" s="256"/>
-      <c r="B188" s="236"/>
+      <c r="A188" s="239"/>
+      <c r="B188" s="237"/>
       <c r="C188" s="58" t="s">
         <v>478</v>
       </c>
@@ -34072,8 +34038,8 @@
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A189" s="257"/>
-      <c r="B189" s="237"/>
+      <c r="A189" s="240"/>
+      <c r="B189" s="236"/>
       <c r="C189" s="58" t="s">
         <v>483</v>
       </c>
@@ -34118,7 +34084,7 @@
       <c r="D192" s="104"/>
     </row>
     <row r="193" spans="1:4" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A193" s="240" t="s">
+      <c r="A193" s="243" t="s">
         <v>84</v>
       </c>
       <c r="B193" s="235" t="s">
@@ -34130,8 +34096,8 @@
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A194" s="246"/>
-      <c r="B194" s="236"/>
+      <c r="A194" s="244"/>
+      <c r="B194" s="237"/>
       <c r="C194" s="70" t="s">
         <v>245</v>
       </c>
@@ -34140,8 +34106,8 @@
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A195" s="246"/>
-      <c r="B195" s="236"/>
+      <c r="A195" s="244"/>
+      <c r="B195" s="237"/>
       <c r="C195" s="70">
         <v>10.1</v>
       </c>
@@ -34150,8 +34116,8 @@
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A196" s="246"/>
-      <c r="B196" s="236"/>
+      <c r="A196" s="244"/>
+      <c r="B196" s="237"/>
       <c r="C196" s="70">
         <v>10.199999999999999</v>
       </c>
@@ -34160,8 +34126,8 @@
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A197" s="246"/>
-      <c r="B197" s="236"/>
+      <c r="A197" s="244"/>
+      <c r="B197" s="237"/>
       <c r="C197" s="98" t="s">
         <v>288</v>
       </c>
@@ -34170,8 +34136,8 @@
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A198" s="246"/>
-      <c r="B198" s="236"/>
+      <c r="A198" s="244"/>
+      <c r="B198" s="237"/>
       <c r="C198" s="98" t="s">
         <v>370</v>
       </c>
@@ -34180,8 +34146,8 @@
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A199" s="246"/>
-      <c r="B199" s="236"/>
+      <c r="A199" s="244"/>
+      <c r="B199" s="237"/>
       <c r="C199" s="98" t="s">
         <v>117</v>
       </c>
@@ -34190,8 +34156,8 @@
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A200" s="246"/>
-      <c r="B200" s="236"/>
+      <c r="A200" s="244"/>
+      <c r="B200" s="237"/>
       <c r="C200" s="98" t="s">
         <v>417</v>
       </c>
@@ -34200,8 +34166,8 @@
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A201" s="246"/>
-      <c r="B201" s="236"/>
+      <c r="A201" s="244"/>
+      <c r="B201" s="237"/>
       <c r="C201" s="98" t="s">
         <v>17</v>
       </c>
@@ -34210,8 +34176,8 @@
       </c>
     </row>
     <row r="202" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A202" s="241"/>
-      <c r="B202" s="237"/>
+      <c r="A202" s="245"/>
+      <c r="B202" s="236"/>
       <c r="C202" s="98" t="s">
         <v>460</v>
       </c>
@@ -34220,7 +34186,7 @@
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A203" s="240" t="s">
+      <c r="A203" s="243" t="s">
         <v>246</v>
       </c>
       <c r="B203" s="235" t="s">
@@ -34232,8 +34198,8 @@
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A204" s="246"/>
-      <c r="B204" s="236"/>
+      <c r="A204" s="244"/>
+      <c r="B204" s="237"/>
       <c r="C204" s="125" t="s">
         <v>428</v>
       </c>
@@ -34264,7 +34230,7 @@
       <c r="D206" s="127"/>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A207" s="240" t="s">
+      <c r="A207" s="243" t="s">
         <v>58</v>
       </c>
       <c r="B207" s="235" t="s">
@@ -34278,8 +34244,8 @@
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A208" s="246"/>
-      <c r="B208" s="236"/>
+      <c r="A208" s="244"/>
+      <c r="B208" s="237"/>
       <c r="C208" s="128" t="s">
         <v>260</v>
       </c>
@@ -34288,15 +34254,15 @@
       </c>
     </row>
     <row r="209" spans="1:4" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A209" s="241"/>
-      <c r="B209" s="237"/>
+      <c r="A209" s="245"/>
+      <c r="B209" s="236"/>
       <c r="C209" s="106"/>
       <c r="D209" s="106" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A210" s="261" t="s">
+      <c r="A210" s="241" t="s">
         <v>59</v>
       </c>
       <c r="B210" s="235" t="s">
@@ -34310,15 +34276,15 @@
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A211" s="262"/>
-      <c r="B211" s="237"/>
+      <c r="A211" s="242"/>
+      <c r="B211" s="236"/>
       <c r="C211" s="118"/>
       <c r="D211" s="106" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A212" s="261" t="s">
+      <c r="A212" s="241" t="s">
         <v>286</v>
       </c>
       <c r="B212" s="235" t="s">
@@ -34330,15 +34296,15 @@
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A213" s="262"/>
-      <c r="B213" s="237"/>
+      <c r="A213" s="242"/>
+      <c r="B213" s="236"/>
       <c r="C213" s="106"/>
       <c r="D213" s="106" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A214" s="261" t="s">
+      <c r="A214" s="241" t="s">
         <v>60</v>
       </c>
       <c r="B214" s="235" t="s">
@@ -34352,8 +34318,8 @@
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A215" s="262"/>
-      <c r="B215" s="237"/>
+      <c r="A215" s="242"/>
+      <c r="B215" s="236"/>
       <c r="C215" s="106"/>
       <c r="D215" s="106" t="s">
         <v>408</v>
@@ -34956,10 +34922,10 @@
       <c r="D265" s="173"/>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A266" s="201" t="s">
+      <c r="A266" s="196" t="s">
         <v>499</v>
       </c>
-      <c r="B266" s="221" t="s">
+      <c r="B266" s="230" t="s">
         <v>432</v>
       </c>
       <c r="C266" s="168" t="s">
@@ -34970,8 +34936,8 @@
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A267" s="201"/>
-      <c r="B267" s="221"/>
+      <c r="A267" s="196"/>
+      <c r="B267" s="230"/>
       <c r="C267" s="168" t="s">
         <v>535</v>
       </c>
@@ -34994,10 +34960,10 @@
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A269" s="212" t="s">
+      <c r="A269" s="201" t="s">
         <v>540</v>
       </c>
-      <c r="B269" s="258" t="s">
+      <c r="B269" s="231" t="s">
         <v>432</v>
       </c>
       <c r="C269" s="168" t="s">
@@ -35008,8 +34974,8 @@
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A270" s="213"/>
-      <c r="B270" s="259"/>
+      <c r="A270" s="202"/>
+      <c r="B270" s="232"/>
       <c r="C270" s="168" t="s">
         <v>543</v>
       </c>
@@ -35320,7 +35286,7 @@
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A293" s="181" t="s">
+      <c r="A293" s="262" t="s">
         <v>579</v>
       </c>
       <c r="B293" s="180" t="s">
@@ -35347,75 +35313,8 @@
         <v>578</v>
       </c>
     </row>
-    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A295" s="126" t="s">
-        <v>581</v>
-      </c>
-      <c r="B295" s="263"/>
-      <c r="C295" s="264"/>
-      <c r="D295" s="264"/>
-    </row>
-    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A296" s="95" t="s">
-        <v>582</v>
-      </c>
-      <c r="B296" s="266" t="s">
-        <v>583</v>
-      </c>
-      <c r="C296" s="265" t="s">
-        <v>584</v>
-      </c>
-      <c r="D296" s="95" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="298" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B298" s="267"/>
-    </row>
   </sheetData>
   <mergeCells count="58">
-    <mergeCell ref="A269:A270"/>
-    <mergeCell ref="B269:B270"/>
-    <mergeCell ref="A266:A267"/>
-    <mergeCell ref="B266:B267"/>
-    <mergeCell ref="A62:A63"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="B136:B186"/>
-    <mergeCell ref="A136:A186"/>
-    <mergeCell ref="A214:A215"/>
-    <mergeCell ref="B214:B215"/>
-    <mergeCell ref="A210:A211"/>
-    <mergeCell ref="B210:B211"/>
-    <mergeCell ref="A212:A213"/>
-    <mergeCell ref="B212:B213"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="A207:A209"/>
-    <mergeCell ref="B207:B209"/>
-    <mergeCell ref="A193:A202"/>
-    <mergeCell ref="B193:B202"/>
-    <mergeCell ref="A65:A77"/>
-    <mergeCell ref="B65:B77"/>
-    <mergeCell ref="A78:A95"/>
-    <mergeCell ref="B78:B95"/>
-    <mergeCell ref="A203:A204"/>
-    <mergeCell ref="B203:B204"/>
-    <mergeCell ref="B187:B189"/>
-    <mergeCell ref="A187:A189"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="C98:C99"/>
-    <mergeCell ref="A96:A109"/>
-    <mergeCell ref="B96:B109"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="A128:A134"/>
-    <mergeCell ref="B128:B134"/>
-    <mergeCell ref="A114:A118"/>
-    <mergeCell ref="B114:B118"/>
-    <mergeCell ref="A121:A127"/>
-    <mergeCell ref="B121:B127"/>
-    <mergeCell ref="C96:C97"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="A13:A18"/>
@@ -35432,6 +35331,48 @@
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="A27:A32"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="C98:C99"/>
+    <mergeCell ref="A96:A109"/>
+    <mergeCell ref="B96:B109"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="A128:A134"/>
+    <mergeCell ref="B128:B134"/>
+    <mergeCell ref="A114:A118"/>
+    <mergeCell ref="B114:B118"/>
+    <mergeCell ref="A121:A127"/>
+    <mergeCell ref="B121:B127"/>
+    <mergeCell ref="C96:C97"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="A207:A209"/>
+    <mergeCell ref="B207:B209"/>
+    <mergeCell ref="A193:A202"/>
+    <mergeCell ref="B193:B202"/>
+    <mergeCell ref="A65:A77"/>
+    <mergeCell ref="B65:B77"/>
+    <mergeCell ref="A78:A95"/>
+    <mergeCell ref="B78:B95"/>
+    <mergeCell ref="A203:A204"/>
+    <mergeCell ref="B203:B204"/>
+    <mergeCell ref="B187:B189"/>
+    <mergeCell ref="A187:A189"/>
+    <mergeCell ref="A269:A270"/>
+    <mergeCell ref="B269:B270"/>
+    <mergeCell ref="A266:A267"/>
+    <mergeCell ref="B266:B267"/>
+    <mergeCell ref="A62:A63"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="B136:B186"/>
+    <mergeCell ref="A136:A186"/>
+    <mergeCell ref="A214:A215"/>
+    <mergeCell ref="B214:B215"/>
+    <mergeCell ref="A210:A211"/>
+    <mergeCell ref="B210:B211"/>
+    <mergeCell ref="A212:A213"/>
+    <mergeCell ref="B212:B213"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>